<commit_message>
Update Telegram lesson links for PL-004 and PL-005
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -459,7 +459,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -752,7 +752,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -806,7 +806,7 @@
               </a:defRPr>
             </a:pPr>
             <a:r>
-              <a:t/>
+              <a:t>None</a:t>
             </a:r>
           </a:p>
         </txPr>
@@ -839,7 +839,7 @@
             </a:defRPr>
           </a:pPr>
           <a:r>
-            <a:t/>
+            <a:t>None</a:t>
           </a:r>
         </a:p>
       </txPr>
@@ -12274,7 +12274,7 @@
       </c>
       <c r="F5" s="45" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf/55</t>
         </is>
       </c>
     </row>
@@ -12306,7 +12306,7 @@
       </c>
       <c r="F6" s="45" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf/60</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add PL-010 (Leica I), extend course to 10 lessons
10 new nodes (PL-HIST-0089..0098) covering the path from the
Ur-Leica prototype and Leica 0-Series to the Leica I launch and
first interchangeable lenses. Flagship: PL-HIST-0092 (Leica I public
debut at the 1925 Leipzig Spring Fair). Telegram link for PL-010
still points to the generic channel, pending the group post URL.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Dashboard" sheetId="1" r:id="R835eaa4126f843b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Master_Facts" sheetId="2" r:id="R3483dfbfc8414c63"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Branches" sheetId="3" r:id="Rfb29fd8fd9b94a10"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Lessons_Map" sheetId="4" r:id="Rdf953e7d2e094497"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Sources" sheetId="5" r:id="Rb175d41dea6c4dee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Lists" sheetId="6" r:id="R69ff9f62362a4fe5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="7" r:id="R289b632f91844611"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Dashboard" sheetId="1" r:id="R89bc147ec81d4166"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Master_Facts" sheetId="2" r:id="Rcae5aa9a01104fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Branches" sheetId="3" r:id="Rfb28ea5c5c7246e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Lessons_Map" sheetId="4" r:id="R41a94ce12af846ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Sources" sheetId="5" r:id="R17f69793fedb41b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Lists" sheetId="6" r:id="R8f7418347b3b429e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="7" r:id="R6823f14f8b7e4aa2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4250,7 +4250,7 @@
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="1"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="37">
+  <x:cellXfs count="41">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="6" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -4355,6 +4355,16 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="7">
@@ -4850,7 +4860,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R69693deb70094111"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9bcb1fa2f44e4f69"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -5063,7 +5073,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="29" t="str">
-        <x:v>PHOTO LAB — Master Timeline v0.6</x:v>
+        <x:v>PHOTO LAB — Master Timeline v0.7</x:v>
       </x:c>
       <x:c r="B1" s="28"/>
       <x:c r="C1" s="28"/>
@@ -5090,7 +5100,7 @@
       </x:c>
       <x:c r="B3" s="33" t="n">
         <x:f>COUNTA('01_Master_Facts'!$A$2:$A$500)</x:f>
-        <x:v>88</x:v>
+        <x:v>98</x:v>
       </x:c>
       <x:c r="C3" s="32" t="s">
         <x:v>4</x:v>
@@ -5104,7 +5114,7 @@
       </x:c>
       <x:c r="B4" s="33" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$N$2:$N$500,5)</x:f>
-        <x:v>37</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="C4" s="32" t="s">
         <x:v>6</x:v>
@@ -5114,11 +5124,11 @@
     </x:row>
     <x:row r="5" ht="15.75" customHeight="1">
       <x:c r="A5" s="32" t="str">
-        <x:v>Узлов для PL-001–PL-009</x:v>
+        <x:v>Узлов для PL-001–PL-010</x:v>
       </x:c>
       <x:c r="B5" s="33" t="n">
-        <x:f>SUM(COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-001"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-002"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-003"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-004"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-005"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-006"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-007"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-008"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-009"))</x:f>
-        <x:v>77</x:v>
+        <x:f>SUM(COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-001"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-002"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-003"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-004"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-005"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-006"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-007"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-008"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-009"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-010"))</x:f>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="C5" s="32" t="str">
         <x:v>Без будущих PL и межурочных узлов</x:v>
@@ -5132,7 +5142,7 @@
       </x:c>
       <x:c r="B6" s="33" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$W$2:$W$500,"&lt;&gt;")</x:f>
-        <x:v>29</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C6" s="32" t="s">
         <x:v>8</x:v>
@@ -5192,7 +5202,7 @@
       </x:c>
       <x:c r="B11" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$H$2:$H$500,A11)</x:f>
-        <x:v>6</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C11" s="28"/>
       <x:c r="D11" s="34" t="s">
@@ -5277,7 +5287,7 @@
       </x:c>
       <x:c r="B16" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$H$2:$H$500,A16)</x:f>
-        <x:v>33</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C16" s="28"/>
       <x:c r="D16" s="34" t="s">
@@ -5332,11 +5342,11 @@
       </x:c>
       <x:c r="C19" s="28"/>
       <x:c r="D19" s="28" t="str">
-        <x:v>будущие PL</x:v>
+        <x:v>PL-010</x:v>
       </x:c>
       <x:c r="E19" s="28" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D19)</x:f>
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15.75" customHeight="1">
@@ -5349,11 +5359,11 @@
       </x:c>
       <x:c r="C20" s="28"/>
       <x:c r="D20" s="28" t="str">
-        <x:v>межурочный узел</x:v>
+        <x:v>будущие PL</x:v>
       </x:c>
       <x:c r="E20" s="28" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D20)</x:f>
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="15.75" customHeight="1">
@@ -5366,11 +5376,11 @@
       </x:c>
       <x:c r="C21" s="28"/>
       <x:c r="D21" s="28" t="str">
-        <x:v>проверить</x:v>
+        <x:v>межурочный узел</x:v>
       </x:c>
       <x:c r="E21" s="28" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D21)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="15.75" customHeight="1">
@@ -5382,8 +5392,13 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C22" s="28"/>
-      <x:c r="D22" s="28"/>
-      <x:c r="E22" s="28"/>
+      <x:c r="D22" s="28" t="str">
+        <x:v>проверить</x:v>
+      </x:c>
+      <x:c r="E22" s="28" t="n">
+        <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D22)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="23" ht="15" customHeight="1">
       <x:c r="A23" s="34"/>
@@ -5428,7 +5443,7 @@
       </x:c>
       <x:c r="B27" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A27)</x:f>
-        <x:v>25</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="C27" s="28"/>
       <x:c r="D27" s="28"/>
@@ -5440,7 +5455,7 @@
       </x:c>
       <x:c r="B28" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A28)</x:f>
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C28" s="28"/>
       <x:c r="D28" s="28"/>
@@ -5476,7 +5491,7 @@
       </x:c>
       <x:c r="B31" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A31)</x:f>
-        <x:v>10</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C31" s="28"/>
       <x:c r="D31" s="28"/>
@@ -5500,7 +5515,7 @@
       </x:c>
       <x:c r="B33" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A33)</x:f>
-        <x:v>13</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="C33" s="28"/>
       <x:c r="D33" s="28"/>
@@ -5524,7 +5539,7 @@
       </x:c>
       <x:c r="B35" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A35)</x:f>
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="C35" s="28"/>
       <x:c r="D35" s="28"/>
@@ -5536,7 +5551,7 @@
       </x:c>
       <x:c r="B36" s="34" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A36)</x:f>
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C36" s="28"/>
       <x:c r="D36" s="28"/>
@@ -5599,7 +5614,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3ef0fb7dbbdf46ec"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd6d48fd5b5524888"/>
 </x:worksheet>
 </file>
 
@@ -12604,16 +12619,802 @@
       </x:c>
       <x:c r="AA89" s="28"/>
     </x:row>
-    <x:row r="90" ht="12.75" customHeight="1"/>
-    <x:row r="91" ht="12.75" customHeight="1"/>
-    <x:row r="92" ht="12.75" customHeight="1"/>
-    <x:row r="93" ht="12.75" customHeight="1"/>
-    <x:row r="94" ht="12.75" customHeight="1"/>
-    <x:row r="95" ht="12.75" customHeight="1"/>
-    <x:row r="96" ht="12.75" customHeight="1"/>
-    <x:row r="97" ht="12.75" customHeight="1"/>
-    <x:row r="98" ht="12.75" customHeight="1"/>
-    <x:row r="99" ht="12.75" customHeight="1"/>
+    <x:row r="90" ht="12.75" customHeight="1">
+      <x:c r="A90" s="28" t="str">
+        <x:v>PL-HIST-0089</x:v>
+      </x:c>
+      <x:c r="B90" s="28" t="str">
+        <x:v>1913–1914</x:v>
+      </x:c>
+      <x:c r="C90" s="28" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D90" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E90" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F90" s="28" t="str">
+        <x:v>Оскар Барнак / Ernst Leitz</x:v>
+      </x:c>
+      <x:c r="G90" s="28" t="str">
+        <x:v>Оскар Барнак создаёт прототип Ur-Leica: компактную камеру под 35-мм киноплёнку, которая станет основой будущей Leica I.</x:v>
+      </x:c>
+      <x:c r="H90" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I90" s="28" t="str">
+        <x:v>Ur-Leica prototype</x:v>
+      </x:c>
+      <x:c r="J90" s="28" t="str">
+        <x:v>Идея 35 мм перестаёт быть только кинематографической: появляется замысел маленькой фотокамеры для серьёзной съёмки.</x:v>
+      </x:c>
+      <x:c r="K90" s="28" t="str">
+        <x:v>35-мм киноплёнка и кадр 24×36</x:v>
+      </x:c>
+      <x:c r="L90" s="28" t="str">
+        <x:v>Leica 0-Series and Leica I</x:v>
+      </x:c>
+      <x:c r="M90" s="28" t="str">
+        <x:v>Переходная технология</x:v>
+      </x:c>
+      <x:c r="N90" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O90" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P90" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="Q90" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="R90" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="S90" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T90" s="28" t="str">
+        <x:v>Для урока важно показать: Leica I родилась не из желания сделать игрушку, а из идеи мобильной серьёзной камеры.</x:v>
+      </x:c>
+      <x:c r="U90" s="28" t="str">
+        <x:v>Маленький прототип на рабочем столе Барнака рядом с полоской 35-мм киноплёнки.</x:v>
+      </x:c>
+      <x:c r="V90" s="28" t="str">
+        <x:v>#PL010 #Ur-Leica #Barnack #Wetzlar #35mm</x:v>
+      </x:c>
+      <x:c r="W90" s="28"/>
+      <x:c r="X90" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y90" s="28" t="str">
+        <x:v>Leica I / прототип</x:v>
+      </x:c>
+      <x:c r="Z90" s="28" t="str">
+        <x:v>Инструмент / устройство</x:v>
+      </x:c>
+      <x:c r="AA90" s="28"/>
+    </x:row>
+    <x:row r="91" ht="12.75" customHeight="1">
+      <x:c r="A91" s="28" t="str">
+        <x:v>PL-HIST-0090</x:v>
+      </x:c>
+      <x:c r="B91" s="28" t="str">
+        <x:v>1923</x:v>
+      </x:c>
+      <x:c r="C91" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D91" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E91" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F91" s="28" t="str">
+        <x:v>Оскар Барнак / Ernst Leitz</x:v>
+      </x:c>
+      <x:c r="G91" s="28" t="str">
+        <x:v>После прототипов появляется проверочная серия Leica 0-Series: небольшая партия камер для испытаний перед коммерческим запуском.</x:v>
+      </x:c>
+      <x:c r="H91" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I91" s="28" t="str">
+        <x:v>Leica 0-Series</x:v>
+      </x:c>
+      <x:c r="J91" s="28" t="str">
+        <x:v>Идея маленькой 35-мм камеры проходит практическую проверку: её нужно не просто изобрести, а сделать пригодной для реальных фотографов.</x:v>
+      </x:c>
+      <x:c r="K91" s="28" t="str">
+        <x:v>Ur-Leica prototype</x:v>
+      </x:c>
+      <x:c r="L91" s="28" t="str">
+        <x:v>Decision to enter serial production</x:v>
+      </x:c>
+      <x:c r="M91" s="28" t="str">
+        <x:v>Переходная технология</x:v>
+      </x:c>
+      <x:c r="N91" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O91" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P91" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="Q91" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="R91" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="S91" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T91" s="28" t="str">
+        <x:v>Хороший storytelling-узел: между прототипом и рынком всегда есть испытание, сомнение и проверка.</x:v>
+      </x:c>
+      <x:c r="U91" s="28" t="str">
+        <x:v>Небольшая партия камер Leica 0-Series на столе в мастерской Leitz.</x:v>
+      </x:c>
+      <x:c r="V91" s="28" t="str">
+        <x:v>#PL010 #Leica0 #preproduction #Leitz #Barnack</x:v>
+      </x:c>
+      <x:c r="W91" s="28" t="str">
+        <x:v>Проверить точное количество камер 0-Series в финальной лекции: источники обычно указывают малую проверочную серию, но формулировки различаются.</x:v>
+      </x:c>
+      <x:c r="X91" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y91" s="28" t="str">
+        <x:v>Leica I / проверочная серия</x:v>
+      </x:c>
+      <x:c r="Z91" s="28" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="AA91" s="28"/>
+    </x:row>
+    <x:row r="92" ht="12.75" customHeight="1">
+      <x:c r="A92" s="28" t="str">
+        <x:v>PL-HIST-0091</x:v>
+      </x:c>
+      <x:c r="B92" s="28" t="str">
+        <x:v>конец 1924</x:v>
+      </x:c>
+      <x:c r="C92" s="28" t="str">
+        <x:v>точная дата</x:v>
+      </x:c>
+      <x:c r="D92" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E92" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F92" s="28" t="str">
+        <x:v>Ernst Leitz II / Ernst Leitz Werke</x:v>
+      </x:c>
+      <x:c r="G92" s="28" t="str">
+        <x:v>Первая серийная версия Leica I официально входит в производство в конце 1924 года, опираясь на опыт Leica 0-Series.</x:v>
+      </x:c>
+      <x:c r="H92" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I92" s="28" t="str">
+        <x:v>Leica I serial production begins</x:v>
+      </x:c>
+      <x:c r="J92" s="28" t="str">
+        <x:v>Leica перестаёт быть лабораторным экспериментом и становится промышленным изделием.</x:v>
+      </x:c>
+      <x:c r="K92" s="28" t="str">
+        <x:v>Leica 0-Series tests</x:v>
+      </x:c>
+      <x:c r="L92" s="28" t="str">
+        <x:v>Public presentation at Leipzig Spring Fair 1925</x:v>
+      </x:c>
+      <x:c r="M92" s="28" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N92" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O92" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P92" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="Q92" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="R92" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="S92" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T92" s="28" t="str">
+        <x:v>Объяснить просто: революция начинается не в момент идеи, а когда идею удалось произвести серийно.</x:v>
+      </x:c>
+      <x:c r="U92" s="28" t="str">
+        <x:v>Фабричная сборка маленьких Leica I в Вецларе, рядом детали корпуса и объектив.</x:v>
+      </x:c>
+      <x:c r="V92" s="28" t="str">
+        <x:v>#PL010 #LeicaI #serial-production #Leitz</x:v>
+      </x:c>
+      <x:c r="W92" s="28"/>
+      <x:c r="X92" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y92" s="28" t="str">
+        <x:v>Leica I / начало производства</x:v>
+      </x:c>
+      <x:c r="Z92" s="28" t="str">
+        <x:v>Распространение / коммерциализация</x:v>
+      </x:c>
+      <x:c r="AA92" s="28"/>
+    </x:row>
+    <x:row r="93" ht="12.75" customHeight="1">
+      <x:c r="A93" s="28" t="str">
+        <x:v>PL-HIST-0092</x:v>
+      </x:c>
+      <x:c r="B93" s="28" t="str">
+        <x:v>1925</x:v>
+      </x:c>
+      <x:c r="C93" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D93" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E93" s="28" t="str">
+        <x:v>Лейпциг</x:v>
+      </x:c>
+      <x:c r="F93" s="28" t="str">
+        <x:v>Ernst Leitz / Leica</x:v>
+      </x:c>
+      <x:c r="G93" s="28" t="str">
+        <x:v>Leica I представлена публике на Лейпцигской весенней ярмарке как первая серийная 35-мм камера Leitz.</x:v>
+      </x:c>
+      <x:c r="H93" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I93" s="28" t="str">
+        <x:v>Leica I at Leipzig Spring Fair</x:v>
+      </x:c>
+      <x:c r="J93" s="28" t="str">
+        <x:v>35 мм получает публичный коммерческий вход в фотографию: маленькая камера становится реальным продуктом.</x:v>
+      </x:c>
+      <x:c r="K93" s="28" t="str">
+        <x:v>Serial production begins at Leitz</x:v>
+      </x:c>
+      <x:c r="L93" s="28" t="str">
+        <x:v>Compact 35 mm photography spreads</x:v>
+      </x:c>
+      <x:c r="M93" s="28" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N93" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O93" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P93" s="28" t="str">
+        <x:v>SRC-063</x:v>
+      </x:c>
+      <x:c r="Q93" s="28" t="str">
+        <x:v>Leica Camera — 100 Years of Leica: Witness to a Century</x:v>
+      </x:c>
+      <x:c r="R93" s="28" t="str">
+        <x:v>https://leica-camera.com/en-GB/press/100-years-leica-witness-century-1925-2025-1</x:v>
+      </x:c>
+      <x:c r="S93" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T93" s="28" t="str">
+        <x:v>Это главный исторический момент урока: Leica I выходит к публике и меняет представление о серьёзной камере.</x:v>
+      </x:c>
+      <x:c r="U93" s="28" t="str">
+        <x:v>Витрина Leica I на ярмарке в Лейпциге; маленькая камера среди больших фотоаппаратов эпохи.</x:v>
+      </x:c>
+      <x:c r="V93" s="28" t="str">
+        <x:v>#PL010 #LeicaI #Leipzig #1925 #35mm-camera</x:v>
+      </x:c>
+      <x:c r="W93" s="28"/>
+      <x:c r="X93" s="28" t="str">
+        <x:v>51.3397, 12.3731</x:v>
+      </x:c>
+      <x:c r="Y93" s="28" t="str">
+        <x:v>Leica I / публичный дебют</x:v>
+      </x:c>
+      <x:c r="Z93" s="28" t="str">
+        <x:v>Ключевой исторический узел</x:v>
+      </x:c>
+      <x:c r="AA93" s="28" t="str">
+        <x:v>да</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="94" ht="12.75" customHeight="1">
+      <x:c r="A94" s="28" t="str">
+        <x:v>PL-HIST-0093</x:v>
+      </x:c>
+      <x:c r="B94" s="28" t="str">
+        <x:v>1925</x:v>
+      </x:c>
+      <x:c r="C94" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D94" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E94" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F94" s="28" t="str">
+        <x:v>Oskar Barnack / Ernst Leitz</x:v>
+      </x:c>
+      <x:c r="G94" s="28" t="str">
+        <x:v>Leica 1(A), разработанная Барнаком, становится первой коммерчески доступной Leica 35-мм камерой и быстро популяризирует 35-мм фотографию.</x:v>
+      </x:c>
+      <x:c r="H94" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I94" s="28" t="str">
+        <x:v>Leica 1(A) 35 mm camera</x:v>
+      </x:c>
+      <x:c r="J94" s="28" t="str">
+        <x:v>Компактность становится серьёзным фотографическим преимуществом: камера теперь может быть постоянно с фотографом.</x:v>
+      </x:c>
+      <x:c r="K94" s="28" t="str">
+        <x:v>Leica I public launch</x:v>
+      </x:c>
+      <x:c r="L94" s="28" t="str">
+        <x:v>New mobile visual practice</x:v>
+      </x:c>
+      <x:c r="M94" s="28" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N94" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O94" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P94" s="28" t="str">
+        <x:v>SRC-064</x:v>
+      </x:c>
+      <x:c r="Q94" s="28" t="str">
+        <x:v>Smithsonian NMAH — Leica 35 mm 1(A) Camera</x:v>
+      </x:c>
+      <x:c r="R94" s="28" t="str">
+        <x:v>https://americanhistory.si.edu/collections/object/nmah_834692</x:v>
+      </x:c>
+      <x:c r="S94" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T94" s="28" t="str">
+        <x:v>Новичку важно понять: Leica I — это не просто новая модель, а изменение поведения фотографа.</x:v>
+      </x:c>
+      <x:c r="U94" s="28" t="str">
+        <x:v>Маленькая Leica I в руке фотографа рядом с большой складной камерой как контраст старого и нового.</x:v>
+      </x:c>
+      <x:c r="V94" s="28" t="str">
+        <x:v>#PL010 #Leica1A #compact-camera #35mm #Barnack</x:v>
+      </x:c>
+      <x:c r="W94" s="28"/>
+      <x:c r="X94" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y94" s="28" t="str">
+        <x:v>Leica I / компактная камера</x:v>
+      </x:c>
+      <x:c r="Z94" s="28" t="str">
+        <x:v>Инструмент / устройство</x:v>
+      </x:c>
+      <x:c r="AA94" s="28"/>
+    </x:row>
+    <x:row r="95" ht="12.75" customHeight="1">
+      <x:c r="A95" s="28" t="str">
+        <x:v>PL-HIST-0094</x:v>
+      </x:c>
+      <x:c r="B95" s="28" t="str">
+        <x:v>1925</x:v>
+      </x:c>
+      <x:c r="C95" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D95" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E95" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F95" s="28" t="str">
+        <x:v>Макс Берек / Leitz</x:v>
+      </x:c>
+      <x:c r="G95" s="28" t="str">
+        <x:v>Первые объективы Leica разрабатывает Макс Берек: 50 мм f/3.5 Anastigmat / Elmax, затем Elmar, чтобы маленький негатив можно было качественно увеличивать.</x:v>
+      </x:c>
+      <x:c r="H95" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I95" s="28" t="str">
+        <x:v>Leica Anastigmat / Elmax / Elmar 50 mm f/3.5</x:v>
+      </x:c>
+      <x:c r="J95" s="28" t="str">
+        <x:v>Малый формат требует сильной оптики: качество объектива становится условием идеи «маленький негатив — большой отпечаток».</x:v>
+      </x:c>
+      <x:c r="K95" s="28" t="str">
+        <x:v>24×36 mm small negative</x:v>
+      </x:c>
+      <x:c r="L95" s="28" t="str">
+        <x:v>Leica becomes practical system for enlargement and printing</x:v>
+      </x:c>
+      <x:c r="M95" s="28" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N95" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O95" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P95" s="28" t="str">
+        <x:v>SRC-065</x:v>
+      </x:c>
+      <x:c r="Q95" s="28" t="str">
+        <x:v>Leica Camera — Understanding Leica Lenses</x:v>
+      </x:c>
+      <x:c r="R95" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/understanding-leica-lenses</x:v>
+      </x:c>
+      <x:c r="S95" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T95" s="28" t="str">
+        <x:v>Это мост к будущим урокам про объективы: формат победил не один, ему понадобилась точная оптика.</x:v>
+      </x:c>
+      <x:c r="U95" s="28" t="str">
+        <x:v>Схема: маленький негатив 24×36 → объектив Elmar → увеличенный отпечаток.</x:v>
+      </x:c>
+      <x:c r="V95" s="28" t="str">
+        <x:v>#PL010 #MaxBerek #Elmar #Leica-lens #small-negative</x:v>
+      </x:c>
+      <x:c r="W95" s="28" t="str">
+        <x:v>Уточнить в финальном тексте различие Anastigmat / Elmax / Elmar, чтобы не смешать ранние версии объектива.</x:v>
+      </x:c>
+      <x:c r="X95" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y95" s="28" t="str">
+        <x:v>Leica I / оптика и Elmar</x:v>
+      </x:c>
+      <x:c r="Z95" s="28" t="str">
+        <x:v>Технология / процесс</x:v>
+      </x:c>
+      <x:c r="AA95" s="28"/>
+    </x:row>
+    <x:row r="96" ht="12.75" customHeight="1">
+      <x:c r="A96" s="28" t="str">
+        <x:v>PL-HIST-0095</x:v>
+      </x:c>
+      <x:c r="B96" s="28" t="str">
+        <x:v>1925–1930</x:v>
+      </x:c>
+      <x:c r="C96" s="28" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D96" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E96" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F96" s="28" t="str">
+        <x:v>Ernst Leitz Werke / пользователи Leica</x:v>
+      </x:c>
+      <x:c r="G96" s="28" t="str">
+        <x:v>За 1925–1930 годы Leica I выпускается десятками тысяч экземпляров в разных вариантах и закрепляет 35-мм компактную камеру как рабочий фотографический инструмент.</x:v>
+      </x:c>
+      <x:c r="H96" s="28" t="str">
+        <x:v>Негатив-позитив</x:v>
+      </x:c>
+      <x:c r="I96" s="28" t="str">
+        <x:v>Leica I mass adoption</x:v>
+      </x:c>
+      <x:c r="J96" s="28" t="str">
+        <x:v>35 мм перестаёт быть нишевым экспериментом и становится устойчивой практикой съёмки.</x:v>
+      </x:c>
+      <x:c r="K96" s="28" t="str">
+        <x:v>Leica I launch</x:v>
+      </x:c>
+      <x:c r="L96" s="28" t="str">
+        <x:v>Global 35 mm compact camera standard</x:v>
+      </x:c>
+      <x:c r="M96" s="28" t="str">
+        <x:v>Распространение / коммерциализация</x:v>
+      </x:c>
+      <x:c r="N96" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O96" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P96" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="Q96" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="R96" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="S96" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T96" s="28" t="str">
+        <x:v>Не перегружать цифрами, но показать масштаб: камера стала не редкостью, а узнаваемым инструментом.</x:v>
+      </x:c>
+      <x:c r="U96" s="28" t="str">
+        <x:v>Ряд Leica I на производственной полке, рядом отметка 1925–1930.</x:v>
+      </x:c>
+      <x:c r="V96" s="28" t="str">
+        <x:v>#PL010 #LeicaI #mass-production #35mm-standard</x:v>
+      </x:c>
+      <x:c r="W96" s="28"/>
+      <x:c r="X96" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y96" s="28" t="str">
+        <x:v>Leica I / массовое принятие</x:v>
+      </x:c>
+      <x:c r="Z96" s="28" t="str">
+        <x:v>Распространение / коммерциализация</x:v>
+      </x:c>
+      <x:c r="AA96" s="28"/>
+    </x:row>
+    <x:row r="97" ht="12.75" customHeight="1">
+      <x:c r="A97" s="28" t="str">
+        <x:v>PL-HIST-0096</x:v>
+      </x:c>
+      <x:c r="B97" s="28" t="str">
+        <x:v>1920-е–1930-е</x:v>
+      </x:c>
+      <x:c r="C97" s="28" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D97" s="28" t="str">
+        <x:v>Европа / США</x:v>
+      </x:c>
+      <x:c r="E97" s="28" t="str">
+        <x:v>распределённый процесс</x:v>
+      </x:c>
+      <x:c r="F97" s="28" t="str">
+        <x:v>Фотографы нового поколения</x:v>
+      </x:c>
+      <x:c r="G97" s="28" t="str">
+        <x:v>Компактная, быстрая и мобильная Leica I помогает сформировать более интимный, спонтанный визуальный язык — основу репортажа и уличной фотографии.</x:v>
+      </x:c>
+      <x:c r="H97" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I97" s="28" t="str">
+        <x:v>Mobile 35 mm visual language</x:v>
+      </x:c>
+      <x:c r="J97" s="28" t="str">
+        <x:v>Фотограф становится менее заметным и быстрее реагирует на жизнь: камера начинает следовать за событием, а не заставлять событие приходить в студию.</x:v>
+      </x:c>
+      <x:c r="K97" s="28" t="str">
+        <x:v>Leica I mass adoption</x:v>
+      </x:c>
+      <x:c r="L97" s="28" t="str">
+        <x:v>Rangefinder and reportage traditions</x:v>
+      </x:c>
+      <x:c r="M97" s="28" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N97" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O97" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P97" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="Q97" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="R97" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="S97" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T97" s="28" t="str">
+        <x:v>Смысл PL-010: Leica изменила не только размер камеры, но и способ видеть — ближе, быстрее, тише.</x:v>
+      </x:c>
+      <x:c r="U97" s="28" t="str">
+        <x:v>Фотограф с маленькой камерой среди городской жизни; люди не позируют, момент происходит сам.</x:v>
+      </x:c>
+      <x:c r="V97" s="28" t="str">
+        <x:v>#PL010 #reportage #street-photography #mobile-camera #visual-language</x:v>
+      </x:c>
+      <x:c r="W97" s="28"/>
+      <x:c r="X97" s="28"/>
+      <x:c r="Y97" s="28" t="str">
+        <x:v>Leica I / новая визуальная практика</x:v>
+      </x:c>
+      <x:c r="Z97" s="28" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="AA97" s="28"/>
+    </x:row>
+    <x:row r="98" ht="12.75" customHeight="1">
+      <x:c r="A98" s="28" t="str">
+        <x:v>PL-HIST-0097</x:v>
+      </x:c>
+      <x:c r="B98" s="28" t="str">
+        <x:v>1930</x:v>
+      </x:c>
+      <x:c r="C98" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D98" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E98" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F98" s="28" t="str">
+        <x:v>Ernst Leitz Werke</x:v>
+      </x:c>
+      <x:c r="G98" s="28" t="str">
+        <x:v>Leica I(C) вводит сменные объективы; к концу 1930 года появляется стандартизированный крепёж, позволяющий использовать объективы с разными камерами Leica 1(C).</x:v>
+      </x:c>
+      <x:c r="H98" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I98" s="28" t="str">
+        <x:v>Leica I(C) interchangeable lenses</x:v>
+      </x:c>
+      <x:c r="J98" s="28" t="str">
+        <x:v>Leica превращается из отдельной камеры в систему: корпус, объективы и аксессуары начинают развиваться вместе.</x:v>
+      </x:c>
+      <x:c r="K98" s="28" t="str">
+        <x:v>Leica I fixed-lens camera</x:v>
+      </x:c>
+      <x:c r="L98" s="28" t="str">
+        <x:v>Leica system and rangefinder cameras</x:v>
+      </x:c>
+      <x:c r="M98" s="28" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="N98" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O98" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P98" s="28" t="str">
+        <x:v>SRC-067</x:v>
+      </x:c>
+      <x:c r="Q98" s="28" t="str">
+        <x:v>Smithsonian NMAH — Leica 1(C)</x:v>
+      </x:c>
+      <x:c r="R98" s="28" t="str">
+        <x:v>https://americanhistory.si.edu/collections/object/nmah_1145349</x:v>
+      </x:c>
+      <x:c r="S98" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T98" s="28" t="str">
+        <x:v>Это не центральный узел PL-010, а мост: после Leica I важной становится идея системы.</x:v>
+      </x:c>
+      <x:c r="U98" s="28" t="str">
+        <x:v>Корпус Leica I(C) и три объектива рядом: 50 мм, широкоугольный и телеобъектив.</x:v>
+      </x:c>
+      <x:c r="V98" s="28" t="str">
+        <x:v>#PL010 #LeicaIC #interchangeable-lenses #Leica-system</x:v>
+      </x:c>
+      <x:c r="W98" s="28" t="str">
+        <x:v>Проверить терминологию крепления: в источниках встречаются screw mount / standardized mount; не называть это байонетом в финальном русском тексте.</x:v>
+      </x:c>
+      <x:c r="X98" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y98" s="28" t="str">
+        <x:v>Leica I / сменные объективы</x:v>
+      </x:c>
+      <x:c r="Z98" s="28" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="AA98" s="28"/>
+    </x:row>
+    <x:row r="99" ht="12.75" customHeight="1">
+      <x:c r="A99" s="28" t="str">
+        <x:v>PL-HIST-0098</x:v>
+      </x:c>
+      <x:c r="B99" s="28" t="str">
+        <x:v>1932</x:v>
+      </x:c>
+      <x:c r="C99" s="28" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D99" s="28" t="str">
+        <x:v>Германия</x:v>
+      </x:c>
+      <x:c r="E99" s="28" t="str">
+        <x:v>Вецлар</x:v>
+      </x:c>
+      <x:c r="F99" s="28" t="str">
+        <x:v>Ernst Leitz Werke</x:v>
+      </x:c>
+      <x:c r="G99" s="28" t="str">
+        <x:v>Leica II становится первой Leica со встроенным дальномером, продолжая линию малой 35-мм камеры в сторону точной быстрой фокусировки.</x:v>
+      </x:c>
+      <x:c r="H99" s="28" t="str">
+        <x:v>Оптические инструменты</x:v>
+      </x:c>
+      <x:c r="I99" s="28" t="str">
+        <x:v>Leica II built-in rangefinder</x:v>
+      </x:c>
+      <x:c r="J99" s="28" t="str">
+        <x:v>Следующий шаг после компактности — скорость и точность наведения: Leica формирует основу дальномерной культуры съёмки.</x:v>
+      </x:c>
+      <x:c r="K99" s="28" t="str">
+        <x:v>Leica I and Leica system</x:v>
+      </x:c>
+      <x:c r="L99" s="28" t="str">
+        <x:v>Future rangefinder photography and Leica M lineage</x:v>
+      </x:c>
+      <x:c r="M99" s="28" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="N99" s="28" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O99" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="P99" s="28" t="str">
+        <x:v>SRC-068</x:v>
+      </x:c>
+      <x:c r="Q99" s="28" t="str">
+        <x:v>Leica Timeline — 1932</x:v>
+      </x:c>
+      <x:c r="R99" s="28" t="str">
+        <x:v>https://timeline.leica-camera.com/en-US/years/1932</x:v>
+      </x:c>
+      <x:c r="S99" s="28" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T99" s="28" t="str">
+        <x:v>Финальный мост урока: PL-010 завершает Модуль 1, но открывает будущие темы про камеры, дальномер и объективы.</x:v>
+      </x:c>
+      <x:c r="U99" s="28" t="str">
+        <x:v>Leica II рядом с Leica I: появляется дальномер как следующий слой управления камерой.</x:v>
+      </x:c>
+      <x:c r="V99" s="28" t="str">
+        <x:v>#PL010 #LeicaII #rangefinder #future-lessons #Leica-system</x:v>
+      </x:c>
+      <x:c r="W99" s="28"/>
+      <x:c r="X99" s="28" t="str">
+        <x:v>50.5619, 8.5044</x:v>
+      </x:c>
+      <x:c r="Y99" s="28" t="str">
+        <x:v>Leica I / мост к дальномерной системе</x:v>
+      </x:c>
+      <x:c r="Z99" s="28" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="AA99" s="28"/>
+    </x:row>
     <x:row r="100" ht="12.75" customHeight="1"/>
     <x:row r="101" ht="12.75" customHeight="1"/>
     <x:row r="102" ht="12.75" customHeight="1"/>
@@ -13054,7 +13855,7 @@
       <x:formula1>'06_Lists'!$E$2:$E$6</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O2:O500">
-      <x:formula1>'06_Lists'!$C$2:$C$13</x:formula1>
+      <x:formula1>'06_Lists'!$C$2:$C$14</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="S2:S500">
       <x:formula1>'06_Lists'!$F$2:$F$6</x:formula1>
@@ -13063,7 +13864,7 @@
       <x:formula1>'06_Lists'!$D$2:$D$14</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Y2:Y500">
-      <x:formula1>'06_Lists'!$H$2:$H$66</x:formula1>
+      <x:formula1>'06_Lists'!$H$2:$H$76</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="Z2:Z500">
       <x:formula1>'06_Lists'!$G$2:$G$11</x:formula1>
@@ -13071,7 +13872,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rabafe04e4bd648ec"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3f890d577a2349a0"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13126,7 +13927,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B3" s="6" t="str">
-        <x:v>camera lucida, stereoscope, portable camera obscura, compact 35mm cameras, Leica system</x:v>
+        <x:v>camera lucida, stereoscope, portable camera obscura, compact 35mm cameras, Leica I, Leica system, rangefinder lineage</x:v>
       </x:c>
       <x:c r="C3" s="6" t="str">
         <x:v>PL-001 / PL-009 / PL-010 / будущие PL</x:v>
@@ -13211,10 +14012,10 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B8" s="6" t="str">
-        <x:v>бумажный негатив, калотип, стеклянный негатив, сухая желатиновая пластина, рулонная плёнка, Brownie, 120 film, 35 мм, 24×36, 135 cartridge, копирование</x:v>
+        <x:v>бумажный негатив, калотип, стеклянный негатив, сухая желатиновая пластина, рулонная плёнка, Brownie, 120 film, 35 мм, 24×36, Leica I, 135 cartridge, копирование</x:v>
       </x:c>
       <x:c r="C8" s="6" t="str">
-        <x:v>PL-004 / PL-006 / PL-007 / PL-008 / PL-009</x:v>
+        <x:v>PL-004 / PL-006 / PL-007 / PL-008 / PL-009 / PL-010</x:v>
       </x:c>
       <x:c r="D8" s="6" t="s">
         <x:v>1224</x:v>
@@ -13328,7 +14129,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re200c697a2e94cf8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R16153f6431224d74"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -13547,26 +14348,46 @@
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="28" t="str">
+        <x:v>PL-010</x:v>
+      </x:c>
+      <x:c r="B11" s="28" t="str">
+        <x:v>Leica I</x:v>
+      </x:c>
+      <x:c r="C11" s="28" t="str">
+        <x:v>PL-HIST-0089…0098</x:v>
+      </x:c>
+      <x:c r="D11" s="28" t="str">
+        <x:v>Leica I сделала 35 мм не просто форматом плёнки, а языком мобильной фотографии: маленькая камера стала серьёзным инструментом репортажа, улицы и повседневного наблюдения.</x:v>
+      </x:c>
+      <x:c r="E11" s="28" t="str">
+        <x:v>основа заполнена</x:v>
+      </x:c>
+      <x:c r="F11" s="28" t="str">
+        <x:v>https://t.me/photolab_vf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="28" t="str">
         <x:v>будущие PL</x:v>
       </x:c>
-      <x:c r="B11" s="28" t="str">
-        <x:v>Расширение после PL-009</x:v>
-      </x:c>
-      <x:c r="C11" s="28" t="str">
-        <x:v>Leica I, цвет, вспышка, автофокус, цифровая фотография, смартфоны, AI</x:v>
-      </x:c>
-      <x:c r="D11" s="28" t="str">
-        <x:v>Фотография станет ещё компактнее, цветной, автоматической, цифровой и вычислительной.</x:v>
-      </x:c>
-      <x:c r="E11" s="28" t="str">
+      <x:c r="B12" s="28" t="str">
+        <x:v>Расширение после PL-010</x:v>
+      </x:c>
+      <x:c r="C12" s="28" t="str">
+        <x:v>Цвет, вспышка, автофокус, цифровая фотография, смартфоны, AI</x:v>
+      </x:c>
+      <x:c r="D12" s="28" t="str">
+        <x:v>После Leica фотография будет развиваться как система: материал, камера, объектив, экспозиция, фокус, жанры, печать и авторский проект.</x:v>
+      </x:c>
+      <x:c r="E12" s="28" t="str">
         <x:v>планируется</x:v>
       </x:c>
-      <x:c r="F11" s="28"/>
+      <x:c r="F12" s="28"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R062f7f485cc64ced"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R53660eaa7e6944b1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14636,10 +15457,129 @@
         <x:v>музейная карточка предмета</x:v>
       </x:c>
     </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="28" t="str">
+        <x:v>SRC-062</x:v>
+      </x:c>
+      <x:c r="B63" s="28" t="str">
+        <x:v>Leica Camera — The History of the Leica I</x:v>
+      </x:c>
+      <x:c r="C63" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/100-years/the-history-of-the-leica-I</x:v>
+      </x:c>
+      <x:c r="D63" s="28" t="str">
+        <x:v>Leica I production, Leipzig 1925, compact mobile camera, around 57,000 units, visual language of reportage and street photography</x:v>
+      </x:c>
+      <x:c r="E63" s="28" t="str">
+        <x:v>официальная история Leica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="28" t="str">
+        <x:v>SRC-063</x:v>
+      </x:c>
+      <x:c r="B64" s="28" t="str">
+        <x:v>Leica Camera — 100 Years of Leica: Witness to a Century</x:v>
+      </x:c>
+      <x:c r="C64" s="28" t="str">
+        <x:v>https://leica-camera.com/en-GB/press/100-years-leica-witness-century-1925-2025-1</x:v>
+      </x:c>
+      <x:c r="D64" s="28" t="str">
+        <x:v>Leica I first series-produced Leica 35mm camera, presented at Leipzig Spring Fair 1925, compact format and new photographic applications</x:v>
+      </x:c>
+      <x:c r="E64" s="28" t="str">
+        <x:v>официальный пресс-материал Leica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="28" t="str">
+        <x:v>SRC-064</x:v>
+      </x:c>
+      <x:c r="B65" s="28" t="str">
+        <x:v>Smithsonian NMAH — Leica 35 mm 1(A) Camera</x:v>
+      </x:c>
+      <x:c r="C65" s="28" t="str">
+        <x:v>https://americanhistory.si.edu/collections/object/nmah_834692</x:v>
+      </x:c>
+      <x:c r="D65" s="28" t="str">
+        <x:v>Leica 1(A), designed by Oskar Barnack, announced 1924, sold 1925, popularized 35mm film photography</x:v>
+      </x:c>
+      <x:c r="E65" s="28" t="str">
+        <x:v>музейная карточка предмета</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="28" t="str">
+        <x:v>SRC-065</x:v>
+      </x:c>
+      <x:c r="B66" s="28" t="str">
+        <x:v>Leica Camera — Understanding Leica Lenses</x:v>
+      </x:c>
+      <x:c r="C66" s="28" t="str">
+        <x:v>https://leica-camera.com/en-int/photography/understanding-leica-lenses</x:v>
+      </x:c>
+      <x:c r="D66" s="28" t="str">
+        <x:v>Max Berek and early Leica lenses for Ur-Leica and Leica system</x:v>
+      </x:c>
+      <x:c r="E66" s="28" t="str">
+        <x:v>официальный материал Leica</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="28" t="str">
+        <x:v>SRC-066</x:v>
+      </x:c>
+      <x:c r="B67" s="28" t="str">
+        <x:v>LFI — Elmar 50 mm f/3.5</x:v>
+      </x:c>
+      <x:c r="C67" s="28" t="str">
+        <x:v>https://lfi-online.de/en/stories/elmar-50-mm-f-3-5-19122.html</x:v>
+      </x:c>
+      <x:c r="D67" s="28" t="str">
+        <x:v>Anastigmat, Elmax and Elmar 50mm f/3.5; Max Berek and early Leica I lenses</x:v>
+      </x:c>
+      <x:c r="E67" s="28" t="str">
+        <x:v>профильный материал Leica Fotografie International</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="A68" s="28" t="str">
+        <x:v>SRC-067</x:v>
+      </x:c>
+      <x:c r="B68" s="28" t="str">
+        <x:v>Smithsonian NMAH — Leica 1(C)</x:v>
+      </x:c>
+      <x:c r="C68" s="28" t="str">
+        <x:v>https://americanhistory.si.edu/collections/object/nmah_1145349</x:v>
+      </x:c>
+      <x:c r="D68" s="28" t="str">
+        <x:v>First Leica with interchangeable lenses in 1930; standardized lens mount by the end of 1930</x:v>
+      </x:c>
+      <x:c r="E68" s="28" t="str">
+        <x:v>музейная карточка предмета</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="A69" s="28" t="str">
+        <x:v>SRC-068</x:v>
+      </x:c>
+      <x:c r="B69" s="28" t="str">
+        <x:v>Leica Timeline — 1932</x:v>
+      </x:c>
+      <x:c r="C69" s="28" t="str">
+        <x:v>https://timeline.leica-camera.com/en-US/years/1932</x:v>
+      </x:c>
+      <x:c r="D69" s="28" t="str">
+        <x:v>Leica II becomes the first Leica with a built-in rangefinder</x:v>
+      </x:c>
+      <x:c r="E69" s="28" t="str">
+        <x:v>официальная история Leica</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R720e8126b0d84c7c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb64bb8c9dd7f4843"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14691,8 +15631,8 @@
       <x:c r="B2" s="6" t="s">
         <x:v>416</x:v>
       </x:c>
-      <x:c r="C2" s="6" t="s">
-        <x:v>13</x:v>
+      <x:c r="C2" s="34" t="str">
+        <x:v>PL-001</x:v>
       </x:c>
       <x:c r="D2" s="6" t="s">
         <x:v>12</x:v>
@@ -14717,8 +15657,8 @@
       <x:c r="B3" s="6" t="s">
         <x:v>328</x:v>
       </x:c>
-      <x:c r="C3" s="6" t="s">
-        <x:v>15</x:v>
+      <x:c r="C3" s="34" t="str">
+        <x:v>PL-002</x:v>
       </x:c>
       <x:c r="D3" s="6" t="s">
         <x:v>14</x:v>
@@ -14743,8 +15683,8 @@
       <x:c r="B4" s="6" t="s">
         <x:v>664</x:v>
       </x:c>
-      <x:c r="C4" s="6" t="s">
-        <x:v>17</x:v>
+      <x:c r="C4" s="34" t="str">
+        <x:v>PL-003</x:v>
       </x:c>
       <x:c r="D4" s="6" t="s">
         <x:v>16</x:v>
@@ -14769,8 +15709,8 @@
       <x:c r="B5" s="6" t="s">
         <x:v>399</x:v>
       </x:c>
-      <x:c r="C5" s="6" t="s">
-        <x:v>19</x:v>
+      <x:c r="C5" s="34" t="str">
+        <x:v>PL-004</x:v>
       </x:c>
       <x:c r="D5" s="6" t="s">
         <x:v>18</x:v>
@@ -14795,8 +15735,8 @@
       <x:c r="B6" s="6" t="s">
         <x:v>756</x:v>
       </x:c>
-      <x:c r="C6" s="6" t="s">
-        <x:v>21</x:v>
+      <x:c r="C6" s="34" t="str">
+        <x:v>PL-005</x:v>
       </x:c>
       <x:c r="D6" s="6" t="s">
         <x:v>20</x:v>
@@ -14819,8 +15759,8 @@
       <x:c r="B7" s="6" t="s">
         <x:v>80</x:v>
       </x:c>
-      <x:c r="C7" s="6" t="s">
-        <x:v>23</x:v>
+      <x:c r="C7" s="34" t="str">
+        <x:v>PL-006</x:v>
       </x:c>
       <x:c r="D7" s="6" t="s">
         <x:v>22</x:v>
@@ -14839,8 +15779,8 @@
       <x:c r="B8" s="6" t="s">
         <x:v>296</x:v>
       </x:c>
-      <x:c r="C8" s="6" t="s">
-        <x:v>25</x:v>
+      <x:c r="C8" s="34" t="str">
+        <x:v>PL-007</x:v>
       </x:c>
       <x:c r="D8" s="6" t="s">
         <x:v>24</x:v>
@@ -14859,8 +15799,8 @@
       <x:c r="B9" s="6" t="s">
         <x:v>555</x:v>
       </x:c>
-      <x:c r="C9" s="6" t="s">
-        <x:v>27</x:v>
+      <x:c r="C9" s="34" t="str">
+        <x:v>PL-008</x:v>
       </x:c>
       <x:c r="D9" s="6" t="s">
         <x:v>26</x:v>
@@ -14879,7 +15819,7 @@
       <x:c r="B10" s="6" t="s">
         <x:v>243</x:v>
       </x:c>
-      <x:c r="C10" s="6" t="str">
+      <x:c r="C10" s="34" t="str">
         <x:v>PL-009</x:v>
       </x:c>
       <x:c r="D10" s="6" t="s">
@@ -14899,8 +15839,8 @@
       <x:c r="B11" s="6" t="s">
         <x:v>206</x:v>
       </x:c>
-      <x:c r="C11" s="6" t="str">
-        <x:v>будущие PL</x:v>
+      <x:c r="C11" s="34" t="str">
+        <x:v>PL-010</x:v>
       </x:c>
       <x:c r="D11" s="6" t="s">
         <x:v>29</x:v>
@@ -14917,8 +15857,8 @@
     <x:row r="12" ht="15.75" customHeight="1">
       <x:c r="A12" s="6"/>
       <x:c r="B12" s="6"/>
-      <x:c r="C12" s="6" t="str">
-        <x:v>межурочный узел</x:v>
+      <x:c r="C12" s="34" t="str">
+        <x:v>будущие PL</x:v>
       </x:c>
       <x:c r="D12" s="6" t="s">
         <x:v>30</x:v>
@@ -14935,8 +15875,8 @@
     <x:row r="13" ht="15.75" customHeight="1">
       <x:c r="A13" s="6"/>
       <x:c r="B13" s="6"/>
-      <x:c r="C13" s="6" t="str">
-        <x:v>проверить</x:v>
+      <x:c r="C13" s="34" t="str">
+        <x:v>межурочный узел</x:v>
       </x:c>
       <x:c r="D13" s="6" t="s">
         <x:v>31</x:v>
@@ -14951,7 +15891,9 @@
     <x:row r="14" ht="15.75" customHeight="1">
       <x:c r="A14" s="6"/>
       <x:c r="B14" s="6"/>
-      <x:c r="C14" s="6"/>
+      <x:c r="C14" s="34" t="str">
+        <x:v>проверить</x:v>
+      </x:c>
       <x:c r="D14" s="6" t="s">
         <x:v>32</x:v>
       </x:c>
@@ -15444,6 +16386,56 @@
     <x:row r="66">
       <x:c r="H66" s="28" t="str">
         <x:v>35 мм / 135 cartridge</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="H67" s="28" t="str">
+        <x:v>Leica I / прототип</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68">
+      <x:c r="H68" s="28" t="str">
+        <x:v>Leica I / проверочная серия</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69">
+      <x:c r="H69" s="28" t="str">
+        <x:v>Leica I / начало производства</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="70">
+      <x:c r="H70" s="28" t="str">
+        <x:v>Leica I / публичный дебют</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71">
+      <x:c r="H71" s="28" t="str">
+        <x:v>Leica I / компактная камера</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72">
+      <x:c r="H72" s="28" t="str">
+        <x:v>Leica I / оптика и Elmar</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73">
+      <x:c r="H73" s="28" t="str">
+        <x:v>Leica I / массовое принятие</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74">
+      <x:c r="H74" s="28" t="str">
+        <x:v>Leica I / новая визуальная практика</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="75">
+      <x:c r="H75" s="28" t="str">
+        <x:v>Leica I / сменные объективы</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="76">
+      <x:c r="H76" s="28" t="str">
+        <x:v>Leica I / мост к дальномерной системе</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -15461,7 +16453,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="35" t="str">
-        <x:v>PHOTO LAB — History Map Master v0.6</x:v>
+        <x:v>PHOTO LAB — History Map Master v0.7</x:v>
       </x:c>
       <x:c r="B1" s="28"/>
     </x:row>
@@ -15475,10 +16467,10 @@
     </x:row>
     <x:row r="3" ht="15.75" customHeight="1">
       <x:c r="A3" s="36" t="str">
-        <x:v>Охват v0.6</x:v>
+        <x:v>Охват v0.7</x:v>
       </x:c>
       <x:c r="B3" s="32" t="str">
-        <x:v>От оптических предпосылок камеры-обскуры до мокрого коллодия, сухих желатиновых пластин, рулонной плёнки, Kodak, Brownie, snapshot-культуры и 35-мм малого формата; основа для PL-001–PL-009.</x:v>
+        <x:v>От оптических предпосылок камеры-обскуры до мокрого коллодия, сухих желатиновых пластин, рулонной плёнки, Kodak, Brownie, snapshot-культуры, 35-мм малого формата и Leica I; основа для PL-001–PL-010.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15.75" customHeight="1">
@@ -15510,7 +16502,7 @@
         <x:v>Правило веток</x:v>
       </x:c>
       <x:c r="B7" s="32" t="str">
-        <x:v>Ветка развития = одна из 13 крупных линий из 02_Branches. Для PL-006…PL-009 сухие пластины, рулонная плёнка, Brownie, snapshot-культура и 35 мм пока идут внутри крупных веток «Негатив-позитив», «Печать / тиражирование», «Проекция / распространение» и «Оптические инструменты», а детали фиксируются в подветках.</x:v>
+        <x:v>Ветка развития = одна из 13 крупных линий из 02_Branches. Для PL-006…PL-010 сухие пластины, рулонная плёнка, Brownie, snapshot-культура, 35 мм и Leica I пока идут внутри крупных веток «Негатив-позитив», «Печать / тиражирование», «Проекция / распространение» и «Оптические инструменты», а детали фиксируются в подветках.</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15.75" customHeight="1">
@@ -15518,7 +16510,7 @@
         <x:v>Правило подветок</x:v>
       </x:c>
       <x:c r="B8" s="32" t="str">
-        <x:v>Подветка (детали) = уточнение внутри крупной ветки: химия, камера, распространение, фотокнига, медицинское применение, сухие пластины, рулонная плёнка, Brownie, snapshot-культура, 35 мм и т.п.</x:v>
+        <x:v>Подветка (детали) = уточнение внутри крупной ветки: химия, камера, распространение, фотокнига, медицинское применение, сухие пластины, рулонная плёнка, Brownie, snapshot-культура, 35 мм, Leica I и т.п.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="12.75" customHeight="1">
@@ -15587,26 +16579,34 @@
     </x:row>
     <x:row r="17" ht="28">
       <x:c r="A17" s="28" t="str">
-        <x:v>Правило флагманских узлов</x:v>
+        <x:v>Что изменено в v0.7</x:v>
       </x:c>
       <x:c r="B17" s="28" t="str">
-        <x:v>Колонка «Флагман урока (да/нет)» = ровно один узел на урок, который представляет тему в компактном/обзорном режиме карты (Journey Mode). Значение проставляется вручную автором, не вычисляется автоматически.</x:v>
+        <x:v>Заполнен PL-010: добавлены PL-HIST-0089…0098 по Leica I, Ur-Leica, Leica 0-Series, серийному запуску 1924/1925, публичному дебюту в Лейпциге, оптике Max Berek / Elmar, массовому распространению, новой мобильной визуальной практике, Leica I(C) и мосту к Leica II. Добавлены источники SRC-062…SRC-068 и флагманский узел PL-HIST-0092.</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="14">
       <x:c r="A18" s="28" t="str">
-        <x:v>Ссылка на урок в Telegram</x:v>
+        <x:v>Правило флагманских узлов</x:v>
       </x:c>
       <x:c r="B18" s="28" t="str">
-        <x:v>Колонка F в 03_Lessons_Map сейчас указывает на канал целиком (https://t.me/photolab_vf), т.к. точные номера постов для каждого PL-00X не зафиксированы. Когда номера постов будут известны, заменить на прямые ссылки вида https://t.me/photolab_vf/123 — сайт должен брать значение из этой колонки, не хранить ссылки в коде.</x:v>
+        <x:v>Колонка «Флагман урока (да/нет)» = ровно один узел на урок, который представляет тему в компактном/обзорном режиме карты (Journey Mode). Значение проставляется вручную автором, не вычисляется автоматически.</x:v>
       </x:c>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="28" t="str">
+        <x:v>Ссылка на урок в Telegram</x:v>
+      </x:c>
+      <x:c r="B19" s="28" t="str">
+        <x:v>Колонка F в 03_Lessons_Map сейчас указывает на канал целиком, если точные номера постов для конкретного PL-00X не зафиксированы. Когда номера постов будут известны, заменить на прямые ссылки вида https://t.me/photolab_vf/123 — сайт должен брать значение из этой колонки, не хранить ссылки в коде.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="28" t="str">
         <x:v>Следующий шаг</x:v>
       </x:c>
-      <x:c r="B19" s="28" t="str">
-        <x:v>PL-010 логично строить вокруг Leica I как камеры, которая сделала 35-мм формат полноценным языком мобильной фотографии.</x:v>
+      <x:c r="B20" s="28" t="str">
+        <x:v>PL-011 начинает Модуль 2: плёнка как светочувствительный материал — нужно перейти от исторической камеры Leica к пониманию самой фотоплёнки.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Add PL-017 (слайдовая плёнка), extend course to 17 lessons
11 новых узлов PL-HIST-0165…0175: от Autochrome (1907) до Ektachrome E100
и архивного хранения слайдов. Флагман — PL-HIST-0167 (Kodachrome, 1935).
Добавлены источники SRC-131…142 и строка PL-017 в 03_Lessons_Map.
Узлы PL-001–016 не изменены.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Dashboard" sheetId="1" r:id="R098f4fefea5f4cc1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Master_Facts" sheetId="2" r:id="R5f3a5bd46c744089"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Branches" sheetId="3" r:id="R9a64e19e61714f20"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Lessons_Map" sheetId="4" r:id="Rd57601f432f84380"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Sources" sheetId="5" r:id="Ree9092e357514b39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Lists" sheetId="6" r:id="R3f6baed17f894a74"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="7" r:id="R867ad533b46846b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05_Dashboard" sheetId="1" r:id="R4feec28623bd4783"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_Master_Facts" sheetId="2" r:id="R6d17a2f109a345b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02_Branches" sheetId="3" r:id="R437fc1b3b1104f1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03_Lessons_Map" sheetId="4" r:id="Ra5b5bc7d1d3447d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04_Sources" sheetId="5" r:id="Ra13b0e51596a4895"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06_Lists" sheetId="6" r:id="R5dacadedde4c4179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_README" sheetId="7" r:id="R6dedb731bc8841ae"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -112,7 +112,7 @@
     <x:xf numFmtId="9" fontId="9" fillId="0" borderId="2"/>
     <x:xf numFmtId="0" fontId="9" fillId="0" borderId="2"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="59">
+  <x:cellXfs count="72">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="6" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -278,6 +278,43 @@
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -768,7 +805,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1da690355b344fe3"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Re6b44dfac77641ea"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -985,7 +1022,7 @@
   <x:sheetData>
     <x:row r="1" s="46" customFormat="1" ht="40" customHeight="1">
       <x:c r="A1" s="31" t="str">
-        <x:v>PHOTO LAB — Master Timeline v0.13</x:v>
+        <x:v>PHOTO LAB — Master Timeline v0.14</x:v>
       </x:c>
       <x:c r="B1" s="20" t="n"/>
       <x:c r="C1" s="20" t="n"/>
@@ -1020,7 +1057,7 @@
       </x:c>
       <x:c r="B3" s="55" t="n">
         <x:f>COUNTA('01_Master_Facts'!$A$2:$A$500)</x:f>
-        <x:v>164</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="C3" s="54" t="inlineStr">
         <x:is>
@@ -1038,7 +1075,7 @@
       </x:c>
       <x:c r="B4" s="55" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$N$2:$N$500,5)</x:f>
-        <x:v>73</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="C4" s="54" t="inlineStr">
         <x:is>
@@ -1050,11 +1087,11 @@
     </x:row>
     <x:row r="5" s="46" customFormat="1" ht="21" customHeight="1">
       <x:c r="A5" s="54" t="str">
-        <x:v>Узлов для PL-001–PL-016</x:v>
+        <x:v>Узлов для PL-001–PL-017</x:v>
       </x:c>
       <x:c r="B5" s="55" t="n">
-        <x:f>SUM(COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-001"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-002"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-003"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-004"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-005"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-006"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-007"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-008"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-009"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-010"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-011"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-012"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-013"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-014"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-015"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-016"))</x:f>
-        <x:v>153</x:v>
+        <x:f>SUM(COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-001"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-002"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-003"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-004"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-005"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-006"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-007"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-008"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-009"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-010"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-011"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-012"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-013"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-014"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-015"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-016"),COUNTIF('01_Master_Facts'!$O$2:$O$500,"PL-017"))</x:f>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C5" s="54" t="str">
         <x:v>Без будущих PL и межурочных узлов</x:v>
@@ -1070,7 +1107,7 @@
       </x:c>
       <x:c r="B6" s="55" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$W$2:$W$500,"&lt;&gt;")</x:f>
-        <x:v>52</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="C6" s="54" t="inlineStr">
         <x:is>
@@ -1167,7 +1204,7 @@
       </x:c>
       <x:c r="B12" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$H$2:$H$500,A12)</x:f>
-        <x:v>29</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="C12" s="49" t="n"/>
       <x:c r="D12" s="50" t="inlineStr">
@@ -1356,7 +1393,7 @@
       </x:c>
       <x:c r="B21" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$H$2:$H$500,A21)</x:f>
-        <x:v>11</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="C21" s="49" t="n"/>
       <x:c r="D21" s="49" t="inlineStr">
@@ -1377,7 +1414,7 @@
       </x:c>
       <x:c r="B22" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$H$2:$H$500,A22)</x:f>
-        <x:v>5</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="C22" s="49" t="n"/>
       <x:c r="D22" s="49" t="inlineStr">
@@ -1431,11 +1468,11 @@
       <x:c r="B26" s="50" t="n"/>
       <x:c r="C26" s="49" t="n"/>
       <x:c r="D26" s="49" t="str">
-        <x:v>будущие PL</x:v>
+        <x:v>PL-017</x:v>
       </x:c>
       <x:c r="E26" s="49" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D26)</x:f>
-        <x:v>9</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="27" s="46" customFormat="1" ht="21" customHeight="1">
@@ -1443,11 +1480,11 @@
       <x:c r="B27" s="50"/>
       <x:c r="C27" s="49" t="n"/>
       <x:c r="D27" s="49" t="str">
-        <x:v>межурочный узел</x:v>
+        <x:v>будущие PL</x:v>
       </x:c>
       <x:c r="E27" s="49" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D27)</x:f>
-        <x:v>2</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="28" s="46" customFormat="1" ht="21" customHeight="1">
@@ -1455,11 +1492,11 @@
       <x:c r="B28" s="50"/>
       <x:c r="C28" s="49" t="n"/>
       <x:c r="D28" s="49" t="str">
-        <x:v>проверить</x:v>
+        <x:v>межурочный узел</x:v>
       </x:c>
       <x:c r="E28" s="49" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D28)</x:f>
-        <x:v>0</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="29" s="46" customFormat="1" ht="21" customHeight="1">
@@ -1470,8 +1507,13 @@
         <x:v>Количество узлов</x:v>
       </x:c>
       <x:c r="C29" s="49" t="n"/>
-      <x:c r="D29" s="49" t="n"/>
-      <x:c r="E29" s="49" t="n"/>
+      <x:c r="D29" s="49" t="str">
+        <x:v>проверить</x:v>
+      </x:c>
+      <x:c r="E29" s="49" t="n">
+        <x:f>COUNTIF('01_Master_Facts'!$O$2:$O$500,D29)</x:f>
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
     <x:row r="30" s="46" customFormat="1" ht="21" customHeight="1">
       <x:c r="A30" s="50" t="str">
@@ -1491,7 +1533,7 @@
       </x:c>
       <x:c r="B31" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A31)</x:f>
-        <x:v>58</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="C31" s="49" t="n"/>
       <x:c r="D31" s="49" t="n"/>
@@ -1539,7 +1581,7 @@
       </x:c>
       <x:c r="B35" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A35)</x:f>
-        <x:v>22</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="C35" s="49" t="n"/>
       <x:c r="D35" s="49" t="n"/>
@@ -1563,7 +1605,7 @@
       </x:c>
       <x:c r="B37" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A37)</x:f>
-        <x:v>20</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C37" s="49" t="n"/>
       <x:c r="D37" s="49" t="n"/>
@@ -1587,7 +1629,7 @@
       </x:c>
       <x:c r="B39" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A39)</x:f>
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C39" s="49" t="n"/>
       <x:c r="D39" s="49" t="n"/>
@@ -1599,7 +1641,7 @@
       </x:c>
       <x:c r="B40" s="50" t="n">
         <x:f>COUNTIF('01_Master_Facts'!$Z$2:$Z$500,A40)</x:f>
-        <x:v>14</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C40" s="49" t="n"/>
       <x:c r="D40" s="49" t="n"/>
@@ -1634,7 +1676,7 @@
     <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a64b63413434ff9"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7ed72ac1543f4793"/>
 </x:worksheet>
 </file>
 
@@ -21263,17 +21305,873 @@
       </x:c>
       <x:c r="AA165"/>
     </x:row>
-    <x:row r="166" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="167" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="168" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="169" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="170" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="171" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="172" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="173" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="174" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="175" s="46" customFormat="1" ht="17" customHeight="1"/>
-    <x:row r="176" s="46" customFormat="1" ht="17" customHeight="1"/>
+    <x:row r="166" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A166" s="62" t="str">
+        <x:v>PL-HIST-0165</x:v>
+      </x:c>
+      <x:c r="B166" s="62" t="str">
+        <x:v>1907</x:v>
+      </x:c>
+      <x:c r="C166" s="62" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D166" s="62" t="str">
+        <x:v>Франция</x:v>
+      </x:c>
+      <x:c r="E166" s="62" t="str">
+        <x:v>Лион / Париж</x:v>
+      </x:c>
+      <x:c r="F166" s="62" t="str">
+        <x:v>Огюст и Луи Люмьер</x:v>
+      </x:c>
+      <x:c r="G166" s="62" t="str">
+        <x:v>Autochrome Lumière становится первым практически и коммерчески успешным способом цветной фотографии: изображение получается как прозрачный позитив, который нужно смотреть на просвет.</x:v>
+      </x:c>
+      <x:c r="H166" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I166" s="62" t="str">
+        <x:v>Autochrome Lumière / color transparency plate</x:v>
+      </x:c>
+      <x:c r="J166" s="62" t="str">
+        <x:v>Цвет перестаёт быть ручной раскраской и становится фотографическим результатом, но пока остаётся уникальной прозрачностью, а не тиражируемым негативом.</x:v>
+      </x:c>
+      <x:c r="K166" s="62" t="str">
+        <x:v>Позитив и прямые позитивные процессы в PL-014</x:v>
+      </x:c>
+      <x:c r="L166" s="62" t="str">
+        <x:v>Рулонная цветная реверсивная плёнка и Kodachrome</x:v>
+      </x:c>
+      <x:c r="M166" s="62" t="str">
+        <x:v>Исторически важная ограниченная ветка</x:v>
+      </x:c>
+      <x:c r="N166" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O166" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P166" s="62" t="str">
+        <x:v>SRC-131</x:v>
+      </x:c>
+      <x:c r="Q166" s="62" t="str">
+        <x:v>National Science and Media Museum — A short history of colour photography</x:v>
+      </x:c>
+      <x:c r="R166" s="62" t="str">
+        <x:v>https://www.scienceandmediamuseum.org.uk/objects-and-stories/history-colour-photography</x:v>
+      </x:c>
+      <x:c r="S166" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T166" s="62" t="str">
+        <x:v>Начать урок можно с парадокса: первый успешный массовый цвет был не негативом, а прозрачным позитивом для просмотра на свет.</x:v>
+      </x:c>
+      <x:c r="U166" s="62" t="str">
+        <x:v>Автохромная стеклянная пластина на световом столе; зёрна крахмала как цветной экран.</x:v>
+      </x:c>
+      <x:c r="V166" s="62" t="str">
+        <x:v>#PL017 #Autochrome #colour #transparency #Lumiere</x:v>
+      </x:c>
+      <x:c r="W166" s="62"/>
+      <x:c r="X166" s="62" t="str">
+        <x:v>45.7640, 4.8357</x:v>
+      </x:c>
+      <x:c r="Y166" s="62" t="str">
+        <x:v>Слайдовая плёнка / ранний цветной позитив</x:v>
+      </x:c>
+      <x:c r="Z166" s="62" t="str">
+        <x:v>Ключевой исторический узел</x:v>
+      </x:c>
+      <x:c r="AA166" s="62"/>
+    </x:row>
+    <x:row r="167" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A167" s="62" t="str">
+        <x:v>PL-HIST-0166</x:v>
+      </x:c>
+      <x:c r="B167" s="62" t="str">
+        <x:v>1923</x:v>
+      </x:c>
+      <x:c r="C167" s="62" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D167" s="62" t="str">
+        <x:v>США</x:v>
+      </x:c>
+      <x:c r="E167" s="62" t="str">
+        <x:v>Рочестер, Нью-Йорк</x:v>
+      </x:c>
+      <x:c r="F167" s="62" t="str">
+        <x:v>Eastman Kodak Company</x:v>
+      </x:c>
+      <x:c r="G167" s="62" t="str">
+        <x:v>Kodak вводит 16-мм reversal film на безопасной ацетатной основе вместе с камерой Cine-Kodak и проектором Kodascope.</x:v>
+      </x:c>
+      <x:c r="H167" s="62" t="str">
+        <x:v>Проекция / распространение</x:v>
+      </x:c>
+      <x:c r="I167" s="62" t="str">
+        <x:v>16mm reversal film / projected positive</x:v>
+      </x:c>
+      <x:c r="J167" s="62" t="str">
+        <x:v>Реверсивный материал закрепляет простую логику показа: снятая плёнка после обработки становится позитивом, который можно проецировать.</x:v>
+      </x:c>
+      <x:c r="K167" s="62" t="str">
+        <x:v>Autochrome как ранняя цветная прозрачность</x:v>
+      </x:c>
+      <x:c r="L167" s="62" t="str">
+        <x:v>Kodachrome как цветная реверсивная плёнка</x:v>
+      </x:c>
+      <x:c r="M167" s="62" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="N167" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O167" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P167" s="62" t="str">
+        <x:v>SRC-133</x:v>
+      </x:c>
+      <x:c r="Q167" s="62" t="str">
+        <x:v>Kodak — 100 Years of 16mm Film</x:v>
+      </x:c>
+      <x:c r="R167" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/100-years-of-16mm-film/</x:v>
+      </x:c>
+      <x:c r="S167" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T167" s="62" t="str">
+        <x:v>Это важный мост: слайдовая логика связана не только с фотоальбомом, но и с проектором, показом, лекцией, семейным просмотром.</x:v>
+      </x:c>
+      <x:c r="U167" s="62" t="str">
+        <x:v>Домашний проектор Kodascope, катушка 16 мм и световой конус на экран.</x:v>
+      </x:c>
+      <x:c r="V167" s="62" t="str">
+        <x:v>#PL017 #reversal #16mm #projection #Kodak</x:v>
+      </x:c>
+      <x:c r="W167" s="62"/>
+      <x:c r="X167" s="62" t="str">
+        <x:v>43.1566, -77.6088</x:v>
+      </x:c>
+      <x:c r="Y167" s="62" t="str">
+        <x:v>Слайдовая плёнка / reversal и проекция</x:v>
+      </x:c>
+      <x:c r="Z167" s="62" t="str">
+        <x:v>Связь / переход</x:v>
+      </x:c>
+      <x:c r="AA167" s="62"/>
+    </x:row>
+    <x:row r="168" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A168" s="62" t="str">
+        <x:v>PL-HIST-0167</x:v>
+      </x:c>
+      <x:c r="B168" s="62" t="str">
+        <x:v>1935</x:v>
+      </x:c>
+      <x:c r="C168" s="62" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D168" s="62" t="str">
+        <x:v>США</x:v>
+      </x:c>
+      <x:c r="E168" s="62" t="str">
+        <x:v>Рочестер, Нью-Йорк</x:v>
+      </x:c>
+      <x:c r="F168" s="62" t="str">
+        <x:v>Leopold Mannes, Leopold Godowsky Jr. / Eastman Kodak Company</x:v>
+      </x:c>
+      <x:c r="G168" s="62" t="str">
+        <x:v>Kodak представляет Kodachrome — первый коммерчески успешный любительский цветной фильм, первоначально для 16-мм кино.</x:v>
+      </x:c>
+      <x:c r="H168" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I168" s="62" t="str">
+        <x:v>KODACHROME / color reversal film</x:v>
+      </x:c>
+      <x:c r="J168" s="62" t="str">
+        <x:v>Качественная цветная прозрачность становится промышленным продуктом: слайдовая эстетика начинает входить в массовую и профессиональную культуру.</x:v>
+      </x:c>
+      <x:c r="K168" s="62" t="str">
+        <x:v>Autochrome и ранние цветные прозрачности</x:v>
+      </x:c>
+      <x:c r="L168" s="62" t="str">
+        <x:v>Kodachrome 35 мм для фотокамер и слайдов</x:v>
+      </x:c>
+      <x:c r="M168" s="62" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N168" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O168" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P168" s="62" t="str">
+        <x:v>SRC-134</x:v>
+      </x:c>
+      <x:c r="Q168" s="62" t="str">
+        <x:v>Kodak — History of Film</x:v>
+      </x:c>
+      <x:c r="R168" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/chronology-of-film/</x:v>
+      </x:c>
+      <x:c r="S168" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T168" s="62" t="str">
+        <x:v>Флагман урока: Kodachrome сделал цветной слайд узнаваемым визуальным языком XX века.</x:v>
+      </x:c>
+      <x:c r="U168" s="62" t="str">
+        <x:v>Коробка Kodachrome, цветная прозрачность в рамке и яркий луч проектора.</x:v>
+      </x:c>
+      <x:c r="V168" s="62" t="str">
+        <x:v>#PL017 #Kodachrome #slide-film #color-reversal #Kodak</x:v>
+      </x:c>
+      <x:c r="W168" s="62"/>
+      <x:c r="X168" s="62" t="str">
+        <x:v>43.1566, -77.6088</x:v>
+      </x:c>
+      <x:c r="Y168" s="62" t="str">
+        <x:v>Слайдовая плёнка / Kodachrome</x:v>
+      </x:c>
+      <x:c r="Z168" s="62" t="str">
+        <x:v>Ключевой исторический узел</x:v>
+      </x:c>
+      <x:c r="AA168" s="62" t="str">
+        <x:v>да</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="169" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A169" s="62" t="str">
+        <x:v>PL-HIST-0168</x:v>
+      </x:c>
+      <x:c r="B169" s="62" t="str">
+        <x:v>1936</x:v>
+      </x:c>
+      <x:c r="C169" s="62" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D169" s="62" t="str">
+        <x:v>США / глобально</x:v>
+      </x:c>
+      <x:c r="E169" s="62" t="str">
+        <x:v>Рочестер, Нью-Йорк / фотомагазины</x:v>
+      </x:c>
+      <x:c r="F169" s="62" t="str">
+        <x:v>Eastman Kodak Company</x:v>
+      </x:c>
+      <x:c r="G169" s="62" t="str">
+        <x:v>После 16-мм Kodachrome появляются 35-мм слайды и 8-мм домашнее кино, что переносит цветную реверсивную логику в фотографическую и бытовую практику.</x:v>
+      </x:c>
+      <x:c r="H169" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I169" s="62" t="str">
+        <x:v>35mm Kodachrome slides / 8mm home movies</x:v>
+      </x:c>
+      <x:c r="J169" s="62" t="str">
+        <x:v>Цветной позитив становится не только киноформатом, но и форматом маленькой фотографии: кадр можно монтировать в рамку, смотреть через лупу или проецировать.</x:v>
+      </x:c>
+      <x:c r="K169" s="62" t="str">
+        <x:v>Kodachrome 1935</x:v>
+      </x:c>
+      <x:c r="L169" s="62" t="str">
+        <x:v>Профессиональная и любительская культура цветных слайдов</x:v>
+      </x:c>
+      <x:c r="M169" s="62" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N169" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O169" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P169" s="62" t="str">
+        <x:v>SRC-134</x:v>
+      </x:c>
+      <x:c r="Q169" s="62" t="str">
+        <x:v>Kodak — History of Film</x:v>
+      </x:c>
+      <x:c r="R169" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/chronology-of-film/</x:v>
+      </x:c>
+      <x:c r="S169" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T169" s="62" t="str">
+        <x:v>Связать с PL-009: 35 мм становится не только чёрно-белым и негативным форматом, но и цветным слайдом.</x:v>
+      </x:c>
+      <x:c r="U169" s="62" t="str">
+        <x:v>35-мм слайд в картонной рамке рядом с кассетой плёнки и лупой.</x:v>
+      </x:c>
+      <x:c r="V169" s="62" t="str">
+        <x:v>#PL017 #35mm #slides #Kodachrome #transparency</x:v>
+      </x:c>
+      <x:c r="W169" s="62"/>
+      <x:c r="X169" s="62" t="str">
+        <x:v>43.1566, -77.6088</x:v>
+      </x:c>
+      <x:c r="Y169" s="62" t="str">
+        <x:v>Слайдовая плёнка / 35 мм слайды</x:v>
+      </x:c>
+      <x:c r="Z169" s="62" t="str">
+        <x:v>Распространение / коммерциализация</x:v>
+      </x:c>
+      <x:c r="AA169" s="62"/>
+    </x:row>
+    <x:row r="170" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A170" s="62" t="str">
+        <x:v>PL-HIST-0169</x:v>
+      </x:c>
+      <x:c r="B170" s="62" t="str">
+        <x:v>1930-е – XX век</x:v>
+      </x:c>
+      <x:c r="C170" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D170" s="62" t="str">
+        <x:v>глобально</x:v>
+      </x:c>
+      <x:c r="E170" s="62" t="str">
+        <x:v>распределённый процесс</x:v>
+      </x:c>
+      <x:c r="F170" s="62" t="str">
+        <x:v>Фотографы, редакции, лекторы, семьи</x:v>
+      </x:c>
+      <x:c r="G170" s="62" t="str">
+        <x:v>Цветной слайд закрепляется как позитивная прозрачность: итоговое изображение находится прямо на плёнке и читается при проходящем свете.</x:v>
+      </x:c>
+      <x:c r="H170" s="62" t="str">
+        <x:v>Проекция / распространение</x:v>
+      </x:c>
+      <x:c r="I170" s="62" t="str">
+        <x:v>Mounted slide / transparency viewing</x:v>
+      </x:c>
+      <x:c r="J170" s="62" t="str">
+        <x:v>В отличие от цветного негатива, слайд уже выглядит как готовая картинка: его можно положить на световой стол, рассмотреть в лупу или показать проектором.</x:v>
+      </x:c>
+      <x:c r="K170" s="62" t="str">
+        <x:v>35-мм Kodachrome и культура проекции</x:v>
+      </x:c>
+      <x:c r="L170" s="62" t="str">
+        <x:v>Реверсивный химический процесс</x:v>
+      </x:c>
+      <x:c r="M170" s="62" t="str">
+        <x:v>Главная линия / практическое управление</x:v>
+      </x:c>
+      <x:c r="N170" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O170" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P170" s="62" t="str">
+        <x:v>SRC-139</x:v>
+      </x:c>
+      <x:c r="Q170" s="62" t="str">
+        <x:v>National Archives — Photographs</x:v>
+      </x:c>
+      <x:c r="R170" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/holdings-maintenance/photographs</x:v>
+      </x:c>
+      <x:c r="S170" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T170" s="62" t="str">
+        <x:v>Это центральное отличие для новичка: негатив нужно инвертировать/печатать, а слайд сам является позитивом.</x:v>
+      </x:c>
+      <x:c r="U170" s="62" t="str">
+        <x:v>Световой стол с mounted slides, лупой и проектором на заднем плане.</x:v>
+      </x:c>
+      <x:c r="V170" s="62" t="str">
+        <x:v>#PL017 #slide #transparency #projection #positive</x:v>
+      </x:c>
+      <x:c r="W170" s="62" t="str">
+        <x:v>Найти отдельный музейный источник по культуре слайд-проекций и редакционной работе со слайдами.</x:v>
+      </x:c>
+      <x:c r="X170" s="62"/>
+      <x:c r="Y170" s="62" t="str">
+        <x:v>Слайдовая плёнка / просмотр на просвет</x:v>
+      </x:c>
+      <x:c r="Z170" s="62" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="AA170" s="62"/>
+    </x:row>
+    <x:row r="171" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A171" s="62" t="str">
+        <x:v>PL-HIST-0170</x:v>
+      </x:c>
+      <x:c r="B171" s="62" t="str">
+        <x:v>XX век</x:v>
+      </x:c>
+      <x:c r="C171" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D171" s="62" t="str">
+        <x:v>глобально</x:v>
+      </x:c>
+      <x:c r="E171" s="62" t="str">
+        <x:v>распределённый процесс</x:v>
+      </x:c>
+      <x:c r="F171" s="62" t="str">
+        <x:v>Производители реверсивных материалов и лаборатории</x:v>
+      </x:c>
+      <x:c r="G171" s="62" t="str">
+        <x:v>Реверсивный материал при съёмке в камере после обработки даёт позитив, а не негатив: это и есть базовый принцип slide / transparency film.</x:v>
+      </x:c>
+      <x:c r="H171" s="62" t="str">
+        <x:v>Фотохимия</x:v>
+      </x:c>
+      <x:c r="I171" s="62" t="str">
+        <x:v>Reversal stock / direct positive development</x:v>
+      </x:c>
+      <x:c r="J171" s="62" t="str">
+        <x:v>Маршрут изображения меняется: вместо «негатив → позитив» появляется «экспозиция → реверсивная обработка → готовый позитив на плёнке».</x:v>
+      </x:c>
+      <x:c r="K171" s="62" t="str">
+        <x:v>Негативно-позитивная система PL-013 / PL-016</x:v>
+      </x:c>
+      <x:c r="L171" s="62" t="str">
+        <x:v>Ektachrome и стандартизированный E-6 процесс</x:v>
+      </x:c>
+      <x:c r="M171" s="62" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N171" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O171" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P171" s="62" t="str">
+        <x:v>SRC-137</x:v>
+      </x:c>
+      <x:c r="Q171" s="62" t="str">
+        <x:v>National Archives — Archival Formats: Glossary of Terms</x:v>
+      </x:c>
+      <x:c r="R171" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/formats/glossary.html</x:v>
+      </x:c>
+      <x:c r="S171" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T171" s="62" t="str">
+        <x:v>Объяснять через схему: цветной негатив — матрица для будущего изображения, слайд — само изображение.</x:v>
+      </x:c>
+      <x:c r="U171" s="62" t="str">
+        <x:v>Две дорожки процесса: слева негатив превращается в отпечаток, справа слайд сразу становится позитивом.</x:v>
+      </x:c>
+      <x:c r="V171" s="62" t="str">
+        <x:v>#PL017 #reversal #positive #transparency #process</x:v>
+      </x:c>
+      <x:c r="W171" s="62"/>
+      <x:c r="X171" s="62"/>
+      <x:c r="Y171" s="62" t="str">
+        <x:v>Слайдовая плёнка / reversal-процесс</x:v>
+      </x:c>
+      <x:c r="Z171" s="62" t="str">
+        <x:v>Технология / процесс</x:v>
+      </x:c>
+      <x:c r="AA171" s="62"/>
+    </x:row>
+    <x:row r="172" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A172" s="62" t="str">
+        <x:v>PL-HIST-0171</x:v>
+      </x:c>
+      <x:c r="B172" s="62" t="str">
+        <x:v>1946</x:v>
+      </x:c>
+      <x:c r="C172" s="62" t="str">
+        <x:v>год</x:v>
+      </x:c>
+      <x:c r="D172" s="62" t="str">
+        <x:v>США</x:v>
+      </x:c>
+      <x:c r="E172" s="62" t="str">
+        <x:v>Рочестер, Нью-Йорк</x:v>
+      </x:c>
+      <x:c r="F172" s="62" t="str">
+        <x:v>Eastman Kodak Company</x:v>
+      </x:c>
+      <x:c r="G172" s="62" t="str">
+        <x:v>Kodak выпускает KODAK EKTACHROME Transparency Sheet Film — цветную прозрачную плёнку, которую фотографы могли обрабатывать сами с помощью химических наборов.</x:v>
+      </x:c>
+      <x:c r="H172" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I172" s="62" t="str">
+        <x:v>KODAK EKTACHROME Transparency Sheet Film</x:v>
+      </x:c>
+      <x:c r="J172" s="62" t="str">
+        <x:v>Цветной слайд становится более доступным для контролируемой обработки: Ektachrome отделяется от сложной сервисной модели Kodachrome.</x:v>
+      </x:c>
+      <x:c r="K172" s="62" t="str">
+        <x:v>Kodachrome как промышленный цветной слайд</x:v>
+      </x:c>
+      <x:c r="L172" s="62" t="str">
+        <x:v>Стандартизация Ektachrome и E-6</x:v>
+      </x:c>
+      <x:c r="M172" s="62" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N172" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O172" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P172" s="62" t="str">
+        <x:v>SRC-135</x:v>
+      </x:c>
+      <x:c r="Q172" s="62" t="str">
+        <x:v>Kodak — Milestones</x:v>
+      </x:c>
+      <x:c r="R172" s="62" t="str">
+        <x:v>https://www.kodak.com/en/company/page/milestones/</x:v>
+      </x:c>
+      <x:c r="S172" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T172" s="62" t="str">
+        <x:v>Важно: Ektachrome — это шаг к большей самостоятельности фотографа и лаборатории.</x:v>
+      </x:c>
+      <x:c r="U172" s="62" t="str">
+        <x:v>Листовая Ektachrome, химический набор и проявочный бачок на лабораторном столе.</x:v>
+      </x:c>
+      <x:c r="V172" s="62" t="str">
+        <x:v>#PL017 #Ektachrome #transparency #Kodak #processing</x:v>
+      </x:c>
+      <x:c r="W172" s="62"/>
+      <x:c r="X172" s="62" t="str">
+        <x:v>43.1566, -77.6088</x:v>
+      </x:c>
+      <x:c r="Y172" s="62" t="str">
+        <x:v>Слайдовая плёнка / Ektachrome</x:v>
+      </x:c>
+      <x:c r="Z172" s="62" t="str">
+        <x:v>Распространение / коммерциализация</x:v>
+      </x:c>
+      <x:c r="AA172" s="62"/>
+    </x:row>
+    <x:row r="173" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A173" s="62" t="str">
+        <x:v>PL-HIST-0172</x:v>
+      </x:c>
+      <x:c r="B173" s="62" t="str">
+        <x:v>1970-е – XXI век</x:v>
+      </x:c>
+      <x:c r="C173" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D173" s="62" t="str">
+        <x:v>глобально</x:v>
+      </x:c>
+      <x:c r="E173" s="62" t="str">
+        <x:v>фотолаборатории</x:v>
+      </x:c>
+      <x:c r="F173" s="62" t="str">
+        <x:v>Kodak / фотолаборатории</x:v>
+      </x:c>
+      <x:c r="G173" s="62" t="str">
+        <x:v>Process E-6 закрепляется как стандартная логика обработки современных цветных реверсивных плёнок семейства Ektachrome и совместимых материалов.</x:v>
+      </x:c>
+      <x:c r="H173" s="62" t="str">
+        <x:v>Фотохимия</x:v>
+      </x:c>
+      <x:c r="I173" s="62" t="str">
+        <x:v>E-6 color reversal process</x:v>
+      </x:c>
+      <x:c r="J173" s="62" t="str">
+        <x:v>Слайдовая плёнка получает понятную лабораторную метку: если материал рассчитан на E-6, значит это цветной reversal / slide-процесс.</x:v>
+      </x:c>
+      <x:c r="K173" s="62" t="str">
+        <x:v>Ektachrome как более доступная реверсивная система</x:v>
+      </x:c>
+      <x:c r="L173" s="62" t="str">
+        <x:v>Современные слайдовые материалы и гибридное сканирование</x:v>
+      </x:c>
+      <x:c r="M173" s="62" t="str">
+        <x:v>Главная линия</x:v>
+      </x:c>
+      <x:c r="N173" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O173" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P173" s="62" t="str">
+        <x:v>SRC-138</x:v>
+      </x:c>
+      <x:c r="Q173" s="62" t="str">
+        <x:v>Kodak — EKTACHROME Color Reversal Control Strips Process E-6</x:v>
+      </x:c>
+      <x:c r="R173" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/ektachrome-color-reversal-control-strips/</x:v>
+      </x:c>
+      <x:c r="S173" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T173" s="62" t="str">
+        <x:v>Практическая формула для ученика: C-41 — цветной негатив; E-6 — цветной слайд / reversal.</x:v>
+      </x:c>
+      <x:c r="U173" s="62" t="str">
+        <x:v>Две коробки химии: C-41 и E-6; рядом две полоски плёнки — оранжевый негатив и прозрачный слайд.</x:v>
+      </x:c>
+      <x:c r="V173" s="62" t="str">
+        <x:v>#PL017 #E6 #color-reversal #processing #Ektachrome</x:v>
+      </x:c>
+      <x:c r="W173" s="62" t="str">
+        <x:v>Точную историческую дату введения E-6 при необходимости уточнить отдельно; для урока важнее современная маркировка процесса.</x:v>
+      </x:c>
+      <x:c r="X173" s="62"/>
+      <x:c r="Y173" s="62" t="str">
+        <x:v>Слайдовая плёнка / E-6</x:v>
+      </x:c>
+      <x:c r="Z173" s="62" t="str">
+        <x:v>Технология / процесс</x:v>
+      </x:c>
+      <x:c r="AA173" s="62"/>
+    </x:row>
+    <x:row r="174" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A174" s="62" t="str">
+        <x:v>PL-HIST-0173</x:v>
+      </x:c>
+      <x:c r="B174" s="62" t="str">
+        <x:v>XX–XXI век</x:v>
+      </x:c>
+      <x:c r="C174" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D174" s="62" t="str">
+        <x:v>глобально</x:v>
+      </x:c>
+      <x:c r="E174" s="62" t="str">
+        <x:v>практика фотографов</x:v>
+      </x:c>
+      <x:c r="F174" s="62" t="str">
+        <x:v>Фотографы, лаборатории, производители плёнки</x:v>
+      </x:c>
+      <x:c r="G174" s="62" t="str">
+        <x:v>Слайдовая плёнка требует более точной экспозиции, потому что итоговый позитив находится прямо на плёнке и даёт меньше места для исправления, чем негатив.</x:v>
+      </x:c>
+      <x:c r="H174" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I174" s="62" t="str">
+        <x:v>Slide film exposure precision / narrow exposure range</x:v>
+      </x:c>
+      <x:c r="J174" s="62" t="str">
+        <x:v>Фотограф учится измерять свет внимательнее: ошибка экспозиции видна сразу на самом слайде, а не компенсируется при печати с негатива.</x:v>
+      </x:c>
+      <x:c r="K174" s="62" t="str">
+        <x:v>Цветной негатив с большой практической гибкостью PL-016</x:v>
+      </x:c>
+      <x:c r="L174" s="62" t="str">
+        <x:v>Экспозиционная широта PL-020</x:v>
+      </x:c>
+      <x:c r="M174" s="62" t="str">
+        <x:v>Главная линия / практическое управление</x:v>
+      </x:c>
+      <x:c r="N174" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="O174" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P174" s="62" t="str">
+        <x:v>SRC-141</x:v>
+      </x:c>
+      <x:c r="Q174" s="62" t="str">
+        <x:v>Kodak Moments — Ektachrome 120 FAQs</x:v>
+      </x:c>
+      <x:c r="R174" s="62" t="str">
+        <x:v>https://business.kodakmoments.com/sites/default/files/files/products/Ektachrome_120_FAQs_English.pdf</x:v>
+      </x:c>
+      <x:c r="S174" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="T174" s="62" t="str">
+        <x:v>Это мост к PL-020: слайдовая плёнка идеально объясняет, что такое экспозиционная широта и почему у разных материалов она разная.</x:v>
+      </x:c>
+      <x:c r="U174" s="62" t="str">
+        <x:v>Одна сцена снята на негатив и слайд: у слайда выбитые света и плотные тени показывают меньший запас.</x:v>
+      </x:c>
+      <x:c r="V174" s="62" t="str">
+        <x:v>#PL017 #exposure #latitude #slide-film #Ektachrome</x:v>
+      </x:c>
+      <x:c r="W174" s="62" t="str">
+        <x:v>Формулировать без абсолютов: точная широта зависит от конкретной плёнки и обработки.</x:v>
+      </x:c>
+      <x:c r="X174" s="62"/>
+      <x:c r="Y174" s="62" t="str">
+        <x:v>Слайдовая плёнка / точность экспозиции</x:v>
+      </x:c>
+      <x:c r="Z174" s="62" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="AA174" s="62"/>
+    </x:row>
+    <x:row r="175" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A175" s="62" t="str">
+        <x:v>PL-HIST-0174</x:v>
+      </x:c>
+      <x:c r="B175" s="62" t="str">
+        <x:v>XXI век</x:v>
+      </x:c>
+      <x:c r="C175" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D175" s="62" t="str">
+        <x:v>США / глобально</x:v>
+      </x:c>
+      <x:c r="E175" s="62" t="str">
+        <x:v>Рочестер / современные рынки плёнки</x:v>
+      </x:c>
+      <x:c r="F175" s="62" t="str">
+        <x:v>Kodak / Kodak licensees / современные фотографы</x:v>
+      </x:c>
+      <x:c r="G175" s="62" t="str">
+        <x:v>KODAK EKTACHROME E100 остаётся современным примером слайдовой плёнки: daylight-balanced color reversal film ISO 100, рассчитанная на процесс E-6.</x:v>
+      </x:c>
+      <x:c r="H175" s="62" t="str">
+        <x:v>Цвет</x:v>
+      </x:c>
+      <x:c r="I175" s="62" t="str">
+        <x:v>KODAK EKTACHROME E100 / modern slide film</x:v>
+      </x:c>
+      <x:c r="J175" s="62" t="str">
+        <x:v>Слайдовая плёнка не только исторический материал: она остаётся живым выбором для тех, кому нужен готовый позитив, чистый цвет и характерная визуальная дисциплина.</x:v>
+      </x:c>
+      <x:c r="K175" s="62" t="str">
+        <x:v>E-6 как современный стандарт обработки</x:v>
+      </x:c>
+      <x:c r="L175" s="62" t="str">
+        <x:v>Гибридный путь: слайд → световой стол / скан → печать</x:v>
+      </x:c>
+      <x:c r="M175" s="62" t="str">
+        <x:v>Главная линия / визуальный язык</x:v>
+      </x:c>
+      <x:c r="N175" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O175" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P175" s="62" t="str">
+        <x:v>SRC-140</x:v>
+      </x:c>
+      <x:c r="Q175" s="62" t="str">
+        <x:v>Kodak — EKTACHROME E100 Film</x:v>
+      </x:c>
+      <x:c r="R175" s="62" t="str">
+        <x:v>https://www.kodak.com/en/still-film/product/professional/ektachrome-e100-film/</x:v>
+      </x:c>
+      <x:c r="S175" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T175" s="62" t="str">
+        <x:v>Можно показать современную связь: Ektachrome сегодня — это не массовый семейный материал, а осознанный визуальный выбор.</x:v>
+      </x:c>
+      <x:c r="U175" s="62" t="str">
+        <x:v>Современная коробка Ektachrome E100, mounted slide и сканер/световой стол.</x:v>
+      </x:c>
+      <x:c r="V175" s="62" t="str">
+        <x:v>#PL017 #EktachromeE100 #E6 #slide-film #modern-film</x:v>
+      </x:c>
+      <x:c r="W175" s="62"/>
+      <x:c r="X175" s="62" t="str">
+        <x:v>43.1566, -77.6088</x:v>
+      </x:c>
+      <x:c r="Y175" s="62" t="str">
+        <x:v>Слайдовая плёнка / современный материал</x:v>
+      </x:c>
+      <x:c r="Z175" s="62" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="AA175" s="62"/>
+    </x:row>
+    <x:row r="176" s="46" customFormat="1" ht="17" customHeight="1">
+      <x:c r="A176" s="62" t="str">
+        <x:v>PL-HIST-0175</x:v>
+      </x:c>
+      <x:c r="B176" s="62" t="str">
+        <x:v>XX–XXI век</x:v>
+      </x:c>
+      <x:c r="C176" s="62" t="str">
+        <x:v>диапазон</x:v>
+      </x:c>
+      <x:c r="D176" s="62" t="str">
+        <x:v>глобально</x:v>
+      </x:c>
+      <x:c r="E176" s="62" t="str">
+        <x:v>архивы, музеи, частные коллекции</x:v>
+      </x:c>
+      <x:c r="F176" s="62" t="str">
+        <x:v>Архивисты, музеи, фотографы</x:v>
+      </x:c>
+      <x:c r="G176" s="62" t="str">
+        <x:v>Слайды и прозрачности требуют аккуратного хранения: материалы должны быть архивного качества, а оригиналы лучше защищать от света, тепла и неподходящих оболочек.</x:v>
+      </x:c>
+      <x:c r="H176" s="62" t="str">
+        <x:v>Проекция / распространение</x:v>
+      </x:c>
+      <x:c r="I176" s="62" t="str">
+        <x:v>Transparency preservation / slide archive</x:v>
+      </x:c>
+      <x:c r="J176" s="62" t="str">
+        <x:v>Слайд — это не промежуточная рабочая матрица, а сам оригинальный позитив. Потеря или выцветание слайда означает потерю финального изображения.</x:v>
+      </x:c>
+      <x:c r="K176" s="62" t="str">
+        <x:v>Современная слайдовая плёнка и световой стол</x:v>
+      </x:c>
+      <x:c r="L176" s="62" t="str">
+        <x:v>Будущие уроки о сканировании, хранении и отпечатке</x:v>
+      </x:c>
+      <x:c r="M176" s="62" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="N176" s="62" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="O176" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="P176" s="62" t="str">
+        <x:v>SRC-142</x:v>
+      </x:c>
+      <x:c r="Q176" s="62" t="str">
+        <x:v>National Archives — What is the Best Way to Store Negatives and Transparencies?</x:v>
+      </x:c>
+      <x:c r="R176" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/storage/negatives-transparencies.html</x:v>
+      </x:c>
+      <x:c r="S176" s="62" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="T176" s="62" t="str">
+        <x:v>Финальный вывод: слайдовая плёнка красива, но требует дисциплины не только при съёмке, но и при хранении.</x:v>
+      </x:c>
+      <x:c r="U176" s="62" t="str">
+        <x:v>Архивная коробка с рамками слайдов, перчатки, световой стол и холодное хранилище.</x:v>
+      </x:c>
+      <x:c r="V176" s="62" t="str">
+        <x:v>#PL017 #slides #transparencies #archive #preservation</x:v>
+      </x:c>
+      <x:c r="W176" s="62"/>
+      <x:c r="X176" s="62"/>
+      <x:c r="Y176" s="62" t="str">
+        <x:v>Слайдовая плёнка / хранение и архив</x:v>
+      </x:c>
+      <x:c r="Z176" s="62" t="str">
+        <x:v>Применение / жанр</x:v>
+      </x:c>
+      <x:c r="AA176" s="62"/>
+    </x:row>
     <x:row r="177" s="46" customFormat="1" ht="17" customHeight="1"/>
     <x:row r="178" s="46" customFormat="1" ht="17" customHeight="1"/>
     <x:row r="179" s="46" customFormat="1" ht="17" customHeight="1"/>
@@ -21654,7 +22552,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7808e7c7a4c44a2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6947169601ab4dc3"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -21758,10 +22656,10 @@
         </x:is>
       </x:c>
       <x:c r="B4" s="50" t="str">
-        <x:v>серебряные соли, желатиновые эмульсии, скрытое изображение, проявление, чувствительность, спектральная чувствительность, зерно, цветные слои, color couplers, C-41</x:v>
+        <x:v>серебряные соли, желатиновые эмульсии, скрытое изображение, проявление, чувствительность, спектральная чувствительность, зерно, цветные слои, color couplers, C-41, E-6, reversal-процесс</x:v>
       </x:c>
       <x:c r="C4" s="50" t="str">
-        <x:v>PL-002 / PL-006 / PL-011 / PL-012 / PL-015 / PL-016</x:v>
+        <x:v>PL-002 / PL-006 / PL-011 / PL-012 / PL-015 / PL-016 / PL-017</x:v>
       </x:c>
       <x:c r="D4" s="50" t="str">
         <x:v>жёлтый</x:v>
@@ -21945,15 +22843,11 @@
           <x:t xml:space="preserve">Уникальный позитив</x:t>
         </x:is>
       </x:c>
-      <x:c r="B12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Bayard, ambrotype, tintype, direct positive, instant print</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C12" s="50" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PL-003 / PL-005 / PL-014</x:t>
-        </x:is>
+      <x:c r="B12" s="50" t="str">
+        <x:v>ранний цвет, Autochrome, Kodachrome, Kodacolor, Ektachrome, цветная негативная и слайдовая плёнка, chromogenic print, C-41, E-6</x:v>
+      </x:c>
+      <x:c r="C12" s="50" t="str">
+        <x:v>PL-014 / PL-016 / PL-017 / будущие PL</x:v>
       </x:c>
       <x:c r="D12" s="50" t="inlineStr">
         <x:is>
@@ -21973,10 +22867,10 @@
         </x:is>
       </x:c>
       <x:c r="B13" s="50" t="str">
-        <x:v>ранний цвет, Autochrome, Kodachrome, Kodacolor, цветная негативная плёнка, chromogenic print, C-41</x:v>
+        <x:v>lantern slides, слайды, прозрачности, projected positive, публичный и семейный показ</x:v>
       </x:c>
       <x:c r="C13" s="50" t="str">
-        <x:v>PL-014 / PL-016 / будущие PL</x:v>
+        <x:v>PL-017 / будущие PL</x:v>
       </x:c>
       <x:c r="D13" s="50" t="str">
         <x:v>радужный</x:v>
@@ -22015,7 +22909,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb01cec759f6342d5"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9823732918734044"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -22553,27 +23447,47 @@
       </x:c>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" t="str">
+      <x:c r="A18" s="62" t="str">
+        <x:v>PL-017</x:v>
+      </x:c>
+      <x:c r="B18" s="62" t="str">
+        <x:v>Слайдовая плёнка</x:v>
+      </x:c>
+      <x:c r="C18" s="62" t="str">
+        <x:v>PL-HIST-0165…0175</x:v>
+      </x:c>
+      <x:c r="D18" s="62" t="str">
+        <x:v>Слайдовая плёнка — это позитивная прозрачность: реверсивный процесс даёт готовое изображение прямо на плёнке, поэтому цвет, проекция и экспозиция требуют большей точности.</x:v>
+      </x:c>
+      <x:c r="E18" s="62" t="str">
+        <x:v>основа заполнена</x:v>
+      </x:c>
+      <x:c r="F18" s="62" t="str">
+        <x:v>https://t.me/photolab_vf</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="62" t="str">
         <x:v>будущие PL</x:v>
       </x:c>
-      <x:c r="B18" t="str">
-        <x:v>Расширение после PL-016</x:v>
-      </x:c>
-      <x:c r="C18" t="str">
-        <x:v>Слайдовая плёнка, ISO, зерно, широта</x:v>
-      </x:c>
-      <x:c r="D18" t="str">
-        <x:v>После цветной негативной системы курс переходит к слайдовой плёнке и практическим параметрам материала: ISO, зерно и экспозиционная широта.</x:v>
-      </x:c>
-      <x:c r="E18" t="str">
+      <x:c r="B19" s="62" t="str">
+        <x:v>Расширение после PL-017</x:v>
+      </x:c>
+      <x:c r="C19" s="62" t="str">
+        <x:v>ISO плёнки, зерно, экспозиционная широта</x:v>
+      </x:c>
+      <x:c r="D19" s="62" t="str">
+        <x:v>После слайдовой плёнки курс переходит к практическим параметрам материала: ISO, зерно и экспозиционная широта.</x:v>
+      </x:c>
+      <x:c r="E19" s="62" t="str">
         <x:v>планируется</x:v>
       </x:c>
-      <x:c r="F18"/>
+      <x:c r="F19" s="62"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc1b479904f144245"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rff5932617418405f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -25906,10 +26820,214 @@
         <x:v>архивный консервационный источник</x:v>
       </x:c>
     </x:row>
+    <x:row r="132">
+      <x:c r="A132" s="62" t="str">
+        <x:v>SRC-131</x:v>
+      </x:c>
+      <x:c r="B132" s="62" t="str">
+        <x:v>National Science and Media Museum — A short history of colour photography</x:v>
+      </x:c>
+      <x:c r="C132" s="62" t="str">
+        <x:v>https://www.scienceandmediamuseum.org.uk/objects-and-stories/history-colour-photography</x:v>
+      </x:c>
+      <x:c r="D132" s="62" t="str">
+        <x:v>Lumière Autochrome: first practical/commercially successful colour photography process; commercial production from 1907; Kodachrome as first commercially successful integral tripack system</x:v>
+      </x:c>
+      <x:c r="E132" s="62" t="str">
+        <x:v>музейный образовательный источник</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133">
+      <x:c r="A133" s="62" t="str">
+        <x:v>SRC-132</x:v>
+      </x:c>
+      <x:c r="B133" s="62" t="str">
+        <x:v>The Metropolitan Museum of Art — Original Autochromes Produced Using the First Color Photographic Process</x:v>
+      </x:c>
+      <x:c r="C133" s="62" t="str">
+        <x:v>https://www.metmuseum.org/de/press-releases/original-color-photographs-by-stieglitz-and-steichen-january-25-30-2011-exhibitions</x:v>
+      </x:c>
+      <x:c r="D133" s="62" t="str">
+        <x:v>Autochromes introduced in France in 1907 by Auguste and Louis Lumière; one-of-a-kind color transparencies viewed when backlit</x:v>
+      </x:c>
+      <x:c r="E133" s="62" t="str">
+        <x:v>музейный источник по автохромам</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="134">
+      <x:c r="A134" s="62" t="str">
+        <x:v>SRC-133</x:v>
+      </x:c>
+      <x:c r="B134" s="62" t="str">
+        <x:v>Kodak — 100 Years of 16mm Film</x:v>
+      </x:c>
+      <x:c r="C134" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/100-years-of-16mm-film/</x:v>
+      </x:c>
+      <x:c r="D134" s="62" t="str">
+        <x:v>1923: Kodak made amateur motion pictures practical with 16mm reversal film, Cine-Kodak camera and Kodascope projector; 1935 Kodachrome introduced in 16mm</x:v>
+      </x:c>
+      <x:c r="E134" s="62" t="str">
+        <x:v>официальный исторический источник Kodak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="135">
+      <x:c r="A135" s="62" t="str">
+        <x:v>SRC-134</x:v>
+      </x:c>
+      <x:c r="B135" s="62" t="str">
+        <x:v>Kodak — History of Film</x:v>
+      </x:c>
+      <x:c r="C135" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/chronology-of-film/</x:v>
+      </x:c>
+      <x:c r="D135" s="62" t="str">
+        <x:v>Kodachrome introduced in 1935 as first commercially successful amateur color film, initially 16mm; 35mm slides and 8mm home movies followed in 1936</x:v>
+      </x:c>
+      <x:c r="E135" s="62" t="str">
+        <x:v>официальная хронология Kodak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="136">
+      <x:c r="A136" s="62" t="str">
+        <x:v>SRC-135</x:v>
+      </x:c>
+      <x:c r="B136" s="62" t="str">
+        <x:v>Kodak — Milestones</x:v>
+      </x:c>
+      <x:c r="C136" s="62" t="str">
+        <x:v>https://www.kodak.com/en/company/page/milestones/</x:v>
+      </x:c>
+      <x:c r="D136" s="62" t="str">
+        <x:v>1935 Kodachrome introduced; 1946 Kodak marketed EKTACHROME Transparency Sheet Film, first Kodak color film photographers could process themselves using chemical kits</x:v>
+      </x:c>
+      <x:c r="E136" s="62" t="str">
+        <x:v>официальные вехи Kodak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" s="62" t="str">
+        <x:v>SRC-136</x:v>
+      </x:c>
+      <x:c r="B137" s="62" t="str">
+        <x:v>V&amp;A — Colour photography</x:v>
+      </x:c>
+      <x:c r="C137" s="62" t="str">
+        <x:v>https://www.vam.ac.uk/articles/colour-photography</x:v>
+      </x:c>
+      <x:c r="D137" s="62" t="str">
+        <x:v>Autochrome became widely accessible in 1907; Kodachrome introduced in 35mm format in 1936 and replaced Autochrome as a leading colour process</x:v>
+      </x:c>
+      <x:c r="E137" s="62" t="str">
+        <x:v>музейный обзор истории цветной фотографии</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="138">
+      <x:c r="A138" s="62" t="str">
+        <x:v>SRC-137</x:v>
+      </x:c>
+      <x:c r="B138" s="62" t="str">
+        <x:v>National Archives — Archival Formats: Glossary of Terms</x:v>
+      </x:c>
+      <x:c r="C138" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/formats/glossary.html</x:v>
+      </x:c>
+      <x:c r="D138" s="62" t="str">
+        <x:v>When used in a camera, reversal stock develops into a positive; glossary also distinguishes color negatives with orange masking</x:v>
+      </x:c>
+      <x:c r="E138" s="62" t="str">
+        <x:v>архивный терминологический источник</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="62" t="str">
+        <x:v>SRC-138</x:v>
+      </x:c>
+      <x:c r="B139" s="62" t="str">
+        <x:v>Kodak — EKTACHROME Color Reversal Control Strips Process E-6</x:v>
+      </x:c>
+      <x:c r="C139" s="62" t="str">
+        <x:v>https://www.kodak.com/en/motion/page/ektachrome-color-reversal-control-strips/</x:v>
+      </x:c>
+      <x:c r="D139" s="62" t="str">
+        <x:v>KODAK EKTACHROME control strips monitor processing of color reversal films through Process E-6</x:v>
+      </x:c>
+      <x:c r="E139" s="62" t="str">
+        <x:v>официальный источник Kodak по E-6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="62" t="str">
+        <x:v>SRC-139</x:v>
+      </x:c>
+      <x:c r="B140" s="62" t="str">
+        <x:v>National Archives — Photographs</x:v>
+      </x:c>
+      <x:c r="C140" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/holdings-maintenance/photographs</x:v>
+      </x:c>
+      <x:c r="D140" s="62" t="str">
+        <x:v>NARA holdings include film-based negatives, transparencies and slides; preservation page links them to photographic processes and handling</x:v>
+      </x:c>
+      <x:c r="E140" s="62" t="str">
+        <x:v>архивный консервационный источник</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="62" t="str">
+        <x:v>SRC-140</x:v>
+      </x:c>
+      <x:c r="B141" s="62" t="str">
+        <x:v>Kodak — EKTACHROME E100 Film</x:v>
+      </x:c>
+      <x:c r="C141" s="62" t="str">
+        <x:v>https://www.kodak.com/en/still-film/product/professional/ektachrome-e100-film/</x:v>
+      </x:c>
+      <x:c r="D141" s="62" t="str">
+        <x:v>KODAK EKTACHROME E100 is daylight-balanced color reversal film, ISO 100/21°, designed for E-6 processing</x:v>
+      </x:c>
+      <x:c r="E141" s="62" t="str">
+        <x:v>официальная страница продукта Kodak</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="62" t="str">
+        <x:v>SRC-141</x:v>
+      </x:c>
+      <x:c r="B142" s="62" t="str">
+        <x:v>Kodak Moments — Ektachrome 120 FAQs</x:v>
+      </x:c>
+      <x:c r="C142" s="62" t="str">
+        <x:v>https://business.kodakmoments.com/sites/default/files/files/products/Ektachrome_120_FAQs_English.pdf</x:v>
+      </x:c>
+      <x:c r="D142" s="62" t="str">
+        <x:v>Color reversal film has a much narrower exposure range than negative-working films; transparency itself serves as a color reference for scanning</x:v>
+      </x:c>
+      <x:c r="E142" s="62" t="str">
+        <x:v>официальный/лицензионный справочник Kodak Moments</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="62" t="str">
+        <x:v>SRC-142</x:v>
+      </x:c>
+      <x:c r="B143" s="62" t="str">
+        <x:v>National Archives — What is the Best Way to Store Negatives and Transparencies?</x:v>
+      </x:c>
+      <x:c r="C143" s="62" t="str">
+        <x:v>https://www.archives.gov/preservation/storage/negatives-transparencies.html</x:v>
+      </x:c>
+      <x:c r="D143" s="62" t="str">
+        <x:v>Guidance on storage materials for negatives and transparencies, including PAT-approved papers/plastics and enclosures</x:v>
+      </x:c>
+      <x:c r="E143" s="62" t="str">
+        <x:v>архивный источник по хранению</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc4b10c04987d4abd"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfebf0e29465644bb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -26434,7 +27552,7 @@
       <x:c r="A18" s="4" t="n"/>
       <x:c r="B18" s="4" t="n"/>
       <x:c r="C18" s="50" t="str">
-        <x:v>будущие PL</x:v>
+        <x:v>PL-017</x:v>
       </x:c>
       <x:c r="D18" s="4" t="n"/>
       <x:c r="E18" s="4" t="n"/>
@@ -26450,7 +27568,7 @@
       <x:c r="A19" s="4" t="n"/>
       <x:c r="B19" s="4" t="n"/>
       <x:c r="C19" s="4" t="str">
-        <x:v>межурочный узел</x:v>
+        <x:v>будущие PL</x:v>
       </x:c>
       <x:c r="D19" s="4" t="n"/>
       <x:c r="E19" s="4" t="n"/>
@@ -26466,7 +27584,7 @@
       <x:c r="A20" s="4" t="n"/>
       <x:c r="B20" s="4" t="n"/>
       <x:c r="C20" s="4" t="str">
-        <x:v>проверить</x:v>
+        <x:v>межурочный узел</x:v>
       </x:c>
       <x:c r="D20" s="4" t="n"/>
       <x:c r="E20" s="4" t="n"/>
@@ -26481,7 +27599,9 @@
     <x:row r="21" s="46" customFormat="1" ht="20" customHeight="1">
       <x:c r="A21" s="4" t="n"/>
       <x:c r="B21" s="4" t="n"/>
-      <x:c r="C21" s="4" t="n"/>
+      <x:c r="C21" s="4" t="str">
+        <x:v>проверить</x:v>
+      </x:c>
       <x:c r="D21" s="4" t="n"/>
       <x:c r="E21" s="4" t="n"/>
       <x:c r="F21" s="4" t="n"/>
@@ -27460,7 +28580,37 @@
     </x:row>
     <x:row r="141">
       <x:c r="H141" t="str">
-        <x:v>Цветная негативная плёнка / хранение и архив</x:v>
+        <x:v>Слайдовая плёнка / ранний цветной позитив</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="H142" t="str">
+        <x:v>Слайдовая плёнка / reversal и проекция</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="H143" t="str">
+        <x:v>Слайдовая плёнка / Kodachrome</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="H144" t="str">
+        <x:v>Слайдовая плёнка / Ektachrome</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="H145" t="str">
+        <x:v>Слайдовая плёнка / E-6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="146">
+      <x:c r="H146" t="str">
+        <x:v>Слайдовая плёнка / точность экспозиции</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="147">
+      <x:c r="H147" t="str">
+        <x:v>Слайдовая плёнка / хранение и архив</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27478,7 +28628,7 @@
   <x:sheetData>
     <x:row r="1" s="46" customFormat="1" ht="40" customHeight="1">
       <x:c r="A1" s="32" t="str">
-        <x:v>PHOTO LAB — History Map Master v0.13</x:v>
+        <x:v>PHOTO LAB — History Map Master v0.14</x:v>
       </x:c>
       <x:c r="B1" s="20" t="n"/>
     </x:row>
@@ -27499,7 +28649,7 @@
         <x:v>Охват v0.13</x:v>
       </x:c>
       <x:c r="B3" s="54" t="str">
-        <x:v>От оптических предпосылок камеры-обскуры до Leica I и Модуля 2: плёнка как материал, эмульсия, негатив, позитив, чёрно-белая и цветная негативная плёнка; основа для PL-001–PL-016.</x:v>
+        <x:v>От оптических предпосылок камеры-обскуры до Leica I и Модуля 2: плёнка как материал, эмульсия, негатив, позитив, чёрно-белая, цветная негативная и слайдовая плёнка; основа для PL-001–PL-017.</x:v>
       </x:c>
     </x:row>
     <x:row r="4" s="46" customFormat="1" ht="21" customHeight="1">
@@ -27545,7 +28695,7 @@
         </x:is>
       </x:c>
       <x:c r="B7" s="54" t="str">
-        <x:v>Ветка развития = одна из 13 крупных линий из 02_Branches. Для PL-016 цветная негативная плёнка связана с «Цвет», «Фотохимия», «Негатив-позитив» и «Печать / тиражирование».</x:v>
+        <x:v>Ветка развития = одна из 13 крупных линий из 02_Branches. Для PL-017 слайдовая плёнка связана с «Цвет», «Фотохимия», «Проекция / распространение» и «Уникальный позитив».</x:v>
       </x:c>
     </x:row>
     <x:row r="8" s="46" customFormat="1" ht="21" customHeight="1">
@@ -27555,7 +28705,7 @@
         </x:is>
       </x:c>
       <x:c r="B8" s="54" t="str">
-        <x:v>Подветка (детали) = уточнение внутри крупной ветки: химия, камера, распространение, фотокнига, медицинское применение, сухие пластины, рулонная плёнка, Brownie, 35 мм, Leica I, структура плёнки, эмульсия, негатив/позитив, позитив, чёрно-белая плёнка, цветная негативная плёнка и т.п.</x:v>
+        <x:v>Подветка (детали) = уточнение внутри крупной ветки: химия, камера, распространение, фотокнига, медицинское применение, сухие пластины, рулонная плёнка, Brownie, 35 мм, Leica I, структура плёнки, эмульсия, негатив/позитив, позитив, чёрно-белая плёнка, цветная негативная плёнка, слайдовая плёнка и т.п.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" s="46" customFormat="1" ht="17" customHeight="1">
@@ -27740,11 +28890,23 @@
     </x:row>
     <x:row r="25">
       <x:c r="A25" t="str">
+        <x:v>Что изменено в v0.14</x:v>
+      </x:c>
+      <x:c r="B25" t="str">
+        <x:v>Заполнен PL-017: добавлены PL-HIST-0165…0175 по слайдовой плёнке — Autochrome как ранняя цветная прозрачность, 16-мм reversal, Kodachrome 1935, 35-мм слайды, принцип direct positive, Ektachrome 1946, E-6, точность экспозиции, современный Ektachrome E100 и архивное хранение прозрачностей. Добавлены источники SRC-131…SRC-142 и флагманский узел PL-HIST-0167.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" t="str">
         <x:v>Следующий шаг</x:v>
       </x:c>
-      <x:c r="B25" t="str">
-        <x:v>PL-017: слайдовая плёнка — объяснить цветную позитивную прозрачность, reversal-процесс, точность экспозиции и отличие от цветного негатива.</x:v>
-      </x:c>
+      <x:c r="B26" t="str">
+        <x:v>PL-018: ISO плёнки — объяснить светочувствительность материала, коробочный ISO, экспонометрию, push/pull и практический выбор плёнки под свет.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27"/>
+      <x:c r="B27"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>

<commit_message>
Point all lesson links at the active photolab_vf_pro channel
PL-011…PL-016: восстановлены конкретные ссылки на посты (в master.xlsx
для правки PL-018…020 они откатились к общей ссылке).
PL-017…PL-020: конкретных ссылок нет — общая https://t.me/photolab_vf_pro
вместо неактивного канала https://t.me/photolab_vf.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/master.xlsx
+++ b/data/master.xlsx
@@ -28952,7 +28952,7 @@
       </c>
       <c r="F12" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/145</t>
         </is>
       </c>
     </row>
@@ -28984,7 +28984,7 @@
       </c>
       <c r="F13" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/151</t>
         </is>
       </c>
     </row>
@@ -29016,7 +29016,7 @@
       </c>
       <c r="F14" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/162</t>
         </is>
       </c>
     </row>
@@ -29048,7 +29048,7 @@
       </c>
       <c r="F15" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/168</t>
         </is>
       </c>
     </row>
@@ -29080,7 +29080,7 @@
       </c>
       <c r="F16" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/173</t>
         </is>
       </c>
     </row>
@@ -29112,7 +29112,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro/4/181</t>
         </is>
       </c>
     </row>
@@ -29144,7 +29144,7 @@
       </c>
       <c r="F18" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro</t>
         </is>
       </c>
     </row>
@@ -29176,7 +29176,7 @@
       </c>
       <c r="F19" s="62" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro</t>
         </is>
       </c>
     </row>
@@ -29208,7 +29208,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro</t>
         </is>
       </c>
     </row>
@@ -29240,7 +29240,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://t.me/photolab_vf</t>
+          <t>https://t.me/photolab_vf_pro</t>
         </is>
       </c>
     </row>

</xml_diff>